<commit_message>
Add Collateral Market Value metric (EXP-001) with full YAML calc-engine pipeline
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -484,94 +484,187 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
+        <v>EXP-001</v>
+      </c>
+      <c r="B3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Current market value of all pledged collateral securing a credit exposure, denominated in USD. At the facility level, aggregates across all collateral positions linked to the facility. At the counterparty level, applies the bank's participation percentage (bank_share_pct) to reflect only the bank's proportionate share of collateral coverage. Supports recovery analysis, secured lending assessment, and credit risk mitigation quantification. Data element: Current_valuation_USD. Sourced from L2 Atomic Layer (collateral_snapshot).
+</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Current Collateral Market Value</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each active facility as of the most recent as_of_date, look up all collateral_snapshot records linked to that facility_id and SUM current_valuation_usd across all associated collateral positions.
+</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="J3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each active facility as of the most recent as_of_date, look up all collateral_snapshot records linked to that facility_id and SUM current_valuation_usd across all associated collateral positions.
+</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Current Collateral Market Value (facility)</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Calc</v>
+      </c>
+      <c r="N3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each counterparty, look up all active facilities via facility_master. For each facility, retrieve the bank's participation percentage (bank_share_pct) from facility_lender_allocation and the facility-level current_valuation_usd (summed across all collateral positions). Multiply collateral value by participation percentage to get the bank's attributable share, then SUM across all facilities for the counterparty. Formula: SUM(current_valuation_usd * bank_share_pct / 100) per counterparty_id.
+</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Current Collateral Market Value (counterparty)</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="R3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each L3 desk in enterprise_business_taxonomy, look up all active facilities with a matching lob_segment_id, retrieve their facility-level current collateral market value, and SUM across all facilities for the desk.
+</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Current Collateral Market Value (desk)</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="V3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each L2 portfolio segment, traverse enterprise_business_taxonomy from facility lob_segment_id (L3 desk) up to its parent_segment_id (L2 portfolio). SUM facility-level collateral market values across all facilities belonging to desks within the portfolio.
+</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Current Collateral Market Value (portfolio)</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="Z3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each L1 business segment / department, traverse enterprise_business_taxonomy two levels up from the facility's lob_segment_id (L3 desk → L2 portfolio → L1 business segment). SUM facility-level collateral market values across all facilities within the segment.
+</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Current Collateral Market Value (business_segment)</v>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
         <v>PROF-108</v>
       </c>
-      <c r="B3" t="str" xml:space="preserve">
+      <c r="B4" t="str" xml:space="preserve">
         <v xml:space="preserve">Total interest cost incurred on funding sources attributable to the reporting unit during the period. At facility level, computed as the product of the committed amount, the bank's participation share, and the cost of funds rate. At higher rollup levels, aggregated as the sum of facility-level interest expense.
 </v>
       </c>
-      <c r="C3" t="str">
+      <c r="C4" t="str">
         <v>Interest Expense</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D4" t="str">
         <v>committed_facility_amt × bank_share_pct × cost_of_funds_rate</v>
       </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="I3" t="str">
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="I4" t="str">
         <v>Calc</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J4" t="str">
         <v>committed_facility_amt × bank_share_pct × cost_of_funds_rate</v>
       </c>
-      <c r="K3" t="str">
+      <c r="K4" t="str">
         <v>Interest Expense (facility)</v>
       </c>
-      <c r="L3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Agg</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="L4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="N4" t="str">
         <v>SUM(Facility Interest Expense) per counterparty</v>
       </c>
-      <c r="O3" t="str">
+      <c r="O4" t="str">
         <v>Interest Expense (counterparty)</v>
       </c>
-      <c r="P3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Agg</v>
-      </c>
-      <c r="R3" t="str">
+      <c r="P4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="R4" t="str">
         <v>SUM(Facility Interest Expense) per L3 desk segment</v>
       </c>
-      <c r="S3" t="str">
+      <c r="S4" t="str">
         <v>Interest Expense (desk)</v>
       </c>
-      <c r="T3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="U3" t="str">
-        <v>Agg</v>
-      </c>
-      <c r="V3" t="str">
+      <c r="T4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="V4" t="str">
         <v>SUM(Facility Interest Expense) per L2 portfolio segment</v>
       </c>
-      <c r="W3" t="str">
+      <c r="W4" t="str">
         <v>Interest Expense (portfolio)</v>
       </c>
-      <c r="X3" t="str">
-        <v>Y</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>Agg</v>
-      </c>
-      <c r="Z3" t="str">
+      <c r="X4" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>Agg</v>
+      </c>
+      <c r="Z4" t="str">
         <v>SUM(Facility Interest Expense) per L1 business segment (department)</v>
       </c>
-      <c r="AA3" t="str">
+      <c r="AA4" t="str">
         <v>Interest Expense (business_segment)</v>
       </c>
-      <c r="AB3" t="str">
+      <c r="AB4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix EXP-001 formulas for GSIB fitness: SCD filter, NULL handling, consistent bank-share
- Add is_current_flag = 'Y' on facility_lender_allocation joins (prevent SCD double-counting)
- COALESCE(bank_share_pct, 100.0) to handle missing allocation records
- Apply bank_share_pct consistently across all 5 rollup levels for reconciliation
- Upgrade V03 reconciliation to compare all levels including counterparty
- Clarify description: raw MV pre-haircut, add FR Y-14Q Schedule G reference

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -487,14 +487,14 @@
         <v>EXP-001</v>
       </c>
       <c r="B3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Current market value of all pledged collateral securing a credit exposure, denominated in USD. At the facility level, aggregates across all collateral positions linked to the facility. At the counterparty level, applies the bank's participation percentage (bank_share_pct) to reflect only the bank's proportionate share of collateral coverage. Supports recovery analysis, secured lending assessment, and credit risk mitigation quantification. Data element: Current_valuation_USD. Sourced from L2 Atomic Layer (collateral_snapshot).
+        <v xml:space="preserve">Current market value of all pledged collateral securing a credit exposure, denominated in USD, reflecting the bank's proportionate share (bank_share_pct). At the facility level, aggregates current_valuation_usd across all collateral positions linked to the facility, weighted by the bank's participation percentage from the current lender allocation record. At higher rollup levels (counterparty, desk, portfolio, business segment), values are summed consistently using the same bank-share-weighted facility amounts, ensuring cross-level reconciliation. NOTE: This metric reports raw market value, not haircut-adjusted recognised value per Basel III CRE22 comprehensive approach. For regulatory CRM recognition, apply haircut_pct from collateral_snapshot. Data element: current_valuation_usd. Sourced from L2 Atomic Layer (collateral_snapshot).
 </v>
       </c>
       <c r="C3" t="str">
         <v>Current Collateral Market Value</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility as of the most recent as_of_date, look up all collateral_snapshot records linked to that facility_id and SUM current_valuation_usd across all associated collateral positions.
+        <v xml:space="preserve">For each active facility, SUM current_valuation_usd across all collateral positions, weighted by the bank's current participation share. Formula: SUM(current_valuation_usd) * COALESCE(bank_share_pct, 100) / 100.
 </v>
       </c>
       <c r="E3" t="str">
@@ -510,10 +510,10 @@
         <v>Y</v>
       </c>
       <c r="I3" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="J3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility as of the most recent as_of_date, look up all collateral_snapshot records linked to that facility_id and SUM current_valuation_usd across all associated collateral positions.
+        <v xml:space="preserve">For each active facility, SUM current_valuation_usd across all collateral positions, weighted by the bank's current participation share. Formula: SUM(current_valuation_usd) * COALESCE(bank_share_pct, 100) / 100.
 </v>
       </c>
       <c r="K3" t="str">
@@ -523,10 +523,10 @@
         <v>Y</v>
       </c>
       <c r="M3" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="N3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty, look up all active facilities via facility_master. For each facility, retrieve the bank's participation percentage (bank_share_pct) from facility_lender_allocation and the facility-level current_valuation_usd (summed across all collateral positions). Multiply collateral value by participation percentage to get the bank's attributable share, then SUM across all facilities for the counterparty. Formula: SUM(current_valuation_usd * bank_share_pct / 100) per counterparty_id.
+        <v xml:space="preserve">SUM of bank-share-weighted facility collateral values per counterparty. Formula: SUM(facility_collateral_mv * COALESCE(bank_share_pct, 100) / 100) grouped by counterparty_id.
 </v>
       </c>
       <c r="O3" t="str">
@@ -539,7 +539,7 @@
         <v>Agg</v>
       </c>
       <c r="R3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L3 desk in enterprise_business_taxonomy, look up all active facilities with a matching lob_segment_id, retrieve their facility-level current collateral market value, and SUM across all facilities for the desk.
+        <v xml:space="preserve">SUM of bank-share-weighted facility collateral values per L3 desk segment.
 </v>
       </c>
       <c r="S3" t="str">
@@ -552,7 +552,7 @@
         <v>Agg</v>
       </c>
       <c r="V3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L2 portfolio segment, traverse enterprise_business_taxonomy from facility lob_segment_id (L3 desk) up to its parent_segment_id (L2 portfolio). SUM facility-level collateral market values across all facilities belonging to desks within the portfolio.
+        <v xml:space="preserve">SUM of bank-share-weighted facility collateral values per L2 portfolio segment. Traverses enterprise_business_taxonomy: L3 desk → L2 portfolio (parent_segment_id).
 </v>
       </c>
       <c r="W3" t="str">
@@ -565,7 +565,7 @@
         <v>Agg</v>
       </c>
       <c r="Z3" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L1 business segment / department, traverse enterprise_business_taxonomy two levels up from the facility's lob_segment_id (L3 desk → L2 portfolio → L1 business segment). SUM facility-level collateral market values across all facilities within the segment.
+        <v xml:space="preserve">SUM of bank-share-weighted facility collateral values per L1 business segment. Traverses enterprise_business_taxonomy: L3 desk → L2 portfolio → L1 segment.
 </v>
       </c>
       <c r="AA3" t="str">

</xml_diff>

<commit_message>
Fix GSIB metric calculators and remediate data gaps
- Correct schema references (l1→l2) across 101 YAML files and Python calculators
  for facility_master, facility_lender_allocation, facility_counterparty_participation
- Rewrite 5 GSIB calculators (Committed/Undrawn/Outstanding Exposure, Interest
  Expense, Interest Income) with proper formulas, date filtering, and participation_pct scaling
- Add filter_by_date() helper in base.py for string vs datetime.date comparison
- Add gap-remediation.ts script that fills missing L2 data (pricing, profitability,
  positions, lender allocation, counterparty participation, taxonomy orphan fixes)
- Fix sql-emitter.ts LOAD_ORDER (l1→l2 for 4 tables)
- All 5 metrics validated: formulas PASS, rollup conservation PASS across all dimensions

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1324,14 +1324,14 @@
         <v>EXP-004</v>
       </c>
       <c r="B12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Total approved committed credit amount in USD representing contractual lending capacity.
+        <v xml:space="preserve">Bank-share-adjusted total approved committed credit amount in USD. Represents the BHC's pro-rata contractual lending capacity per facility. Maps to FR Y-14Q Field 24 (Committed Exposure Global, MDRM G074).
 </v>
       </c>
       <c r="C12" t="str">
         <v>Committed Exposure ($)</v>
       </c>
       <c r="D12" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Distinct([Facility ID]), WHEN IS(MAX(AS_OF_DATE) AND [Facility_Active_Flag]="Y", THEN [Committed_Facility_Amt]*[Bank_Share] == [Committed Exposure, Bank Share portion only]
+        <v xml:space="preserve">For each active facility: committed_facility_amt * bank_share_pct / 100. bank_share_pct sourced from facility_lender_allocation (aggregated per facility).
 </v>
       </c>
       <c r="E12" t="str">
@@ -1350,7 +1350,7 @@
         <v>Calc</v>
       </c>
       <c r="J12" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Distinct([Facility ID]), WHEN IS(MAX(AS_OF_DATE) AND [Facility_Active_Flag]="Y", THEN [Committed_Facility_Amt]*[Bank_Share] == [Committed Exposure, Bank Share portion only]
+        <v xml:space="preserve">For each active facility: committed_facility_amt * bank_share_pct / 100. bank_share_pct sourced from facility_lender_allocation (aggregated per facility).
 </v>
       </c>
       <c r="K12" t="str">
@@ -1363,7 +1363,7 @@
         <v>Agg</v>
       </c>
       <c r="N12" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level committed_facility_amt per counterparty.
+        <v xml:space="preserve">SUM of facility-level committed exposure weighted by participation_pct from facility_counterparty_participation. Uses contractual pro-rata basis per FR Y-14Q requirements.
 </v>
       </c>
       <c r="O12" t="str">
@@ -1376,7 +1376,7 @@
         <v>Agg</v>
       </c>
       <c r="R12" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level committed_facility_amt per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level committed exposure per L3 desk segment. Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
 </v>
       </c>
       <c r="S12" t="str">
@@ -1389,7 +1389,7 @@
         <v>Agg</v>
       </c>
       <c r="V12" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level committed_facility_amt per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level committed exposure per L2 portfolio segment. Traverses L3 -&gt; L2 via parent_segment_id.
 </v>
       </c>
       <c r="W12" t="str">
@@ -1402,7 +1402,7 @@
         <v>Agg</v>
       </c>
       <c r="Z12" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level committed_facility_amt per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level committed exposure per L1 business segment. Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA12" t="str">
@@ -2537,7 +2537,7 @@
         <v>EXP-017</v>
       </c>
       <c r="B25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Bank-share-adjusted unfunded commitment amount. Measures contingent funding risk by summing unfunded positions per facility, applying the bank's share percentage.
+        <v xml:space="preserve">Bank-share-adjusted unfunded commitment amount. Measures contingent funding risk by summing unfunded positions per facility, applying the bank's share percentage from facility_lender_allocation. Derived as Committed Exposure minus Outstanding Exposure.
 </v>
       </c>
       <c r="C25" t="str">
@@ -2545,9 +2545,9 @@
       </c>
       <c r="D25" t="str" xml:space="preserve">
         <v xml:space="preserve">For each active facility:
-1. Join position → position_detail on position_id (both as_of_date filtered)
+1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
 2. SUM(unfunded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 1.0) for bank-share-adjusted exposure
+3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
 </v>
       </c>
       <c r="E25" t="str">
@@ -2567,9 +2567,9 @@
       </c>
       <c r="J25" t="str" xml:space="preserve">
         <v xml:space="preserve">For each active facility:
-1. Join position → position_detail on position_id (both as_of_date filtered)
+1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
 2. SUM(unfunded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 1.0) for bank-share-adjusted exposure
+3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
 </v>
       </c>
       <c r="K25" t="str">
@@ -2597,6 +2597,7 @@
       </c>
       <c r="R25" t="str" xml:space="preserve">
         <v xml:space="preserve">SUM of facility-level undrawn exposure per L3 desk segment.
+Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
 </v>
       </c>
       <c r="S25" t="str">
@@ -2610,6 +2611,7 @@
       </c>
       <c r="V25" t="str" xml:space="preserve">
         <v xml:space="preserve">SUM of facility-level undrawn exposure per L2 portfolio segment.
+Traverses L3 -&gt; L2 via parent_segment_id.
 </v>
       </c>
       <c r="W25" t="str">
@@ -2623,6 +2625,7 @@
       </c>
       <c r="Z25" t="str" xml:space="preserve">
         <v xml:space="preserve">SUM of facility-level undrawn exposure per L1 business segment.
+Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA25" t="str">
@@ -2637,14 +2640,17 @@
         <v>EXP-018</v>
       </c>
       <c r="B26" t="str" xml:space="preserve">
-        <v xml:space="preserve">Portion of committed exposure currently available and not yet drawn. Used to assess funding deployment and credit capacity usage.
+        <v xml:space="preserve">Bank-share-adjusted funded (drawn) exposure amount. Represents the portion of committed credit currently utilized by the borrower. Maps to FR Y-14Q Field 25 (Utilized Exposure Global, MDRM G075).
 </v>
       </c>
       <c r="C26" t="str">
-        <v>Oustanding Exposure ($)</v>
+        <v>Outstanding Exposure ($)</v>
       </c>
       <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Distinct([Facility ID]), WHEN IS(MAX(AS_OF_DATE) AND [Facility_Active_Flag]="Y", THEN Lookup [Position_ID] within Positions table WHEN IS([Facility_ID]) FOR each [Facility_ID] SUM(ARRAY{[funded_amount]} for each [Position_ID]}) * [Bank_Share] == [Facility Oustanding Exposure, Bank Share Only]
+        <v xml:space="preserve">For each active facility:
+1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
+2. SUM(funded_amount) across all positions for the facility
+3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
 </v>
       </c>
       <c r="E26" t="str">
@@ -2663,24 +2669,29 @@
         <v>Calc</v>
       </c>
       <c r="J26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Distinct([Facility ID]), WHEN IS(MAX(AS_OF_DATE) AND [Facility_Active_Flag]="Y", THEN Lookup [Position_ID] within Positions table WHEN IS([Facility_ID]) FOR each [Facility_ID] SUM(ARRAY{[funded_amount]} for each [Position_ID]}) * [Bank_Share] == [Facility Oustanding Exposure, Bank Share Only]
+        <v xml:space="preserve">For each active facility:
+1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
+2. SUM(funded_amount) across all positions for the facility
+3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
 </v>
       </c>
       <c r="K26" t="str">
-        <v>Oustanding Exposure ($) (facility)</v>
+        <v>Outstanding Exposure ($) (facility)</v>
       </c>
       <c r="L26" t="str">
         <v>Y</v>
       </c>
       <c r="M26" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level funded_amount per counterparty.
+        <v xml:space="preserve">For each counterparty, sum facility-level outstanding exposure weighted
+by participation_pct from facility_counterparty_participation.
+Uses contractual pro-rata basis per FR Y-14Q requirements.
 </v>
       </c>
       <c r="O26" t="str">
-        <v>Oustanding Exposure ($) (counterparty)</v>
+        <v>Outstanding Exposure ($) (counterparty)</v>
       </c>
       <c r="P26" t="str">
         <v>Y</v>
@@ -2689,11 +2700,12 @@
         <v>Agg</v>
       </c>
       <c r="R26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level funded_amount per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level outstanding exposure per L3 desk segment.
+Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
 </v>
       </c>
       <c r="S26" t="str">
-        <v>Oustanding Exposure ($) (desk)</v>
+        <v>Outstanding Exposure ($) (desk)</v>
       </c>
       <c r="T26" t="str">
         <v>Y</v>
@@ -2702,11 +2714,12 @@
         <v>Agg</v>
       </c>
       <c r="V26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level funded_amount per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level outstanding exposure per L2 portfolio segment.
+Traverses L3 -&gt; L2 via parent_segment_id.
 </v>
       </c>
       <c r="W26" t="str">
-        <v>Oustanding Exposure ($) (portfolio)</v>
+        <v>Outstanding Exposure ($) (portfolio)</v>
       </c>
       <c r="X26" t="str">
         <v>Y</v>
@@ -2715,11 +2728,12 @@
         <v>Agg</v>
       </c>
       <c r="Z26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level funded_amount per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level outstanding exposure per L1 business segment.
+Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA26" t="str">
-        <v>Oustanding Exposure ($) (business_segment)</v>
+        <v>Outstanding Exposure ($) (business_segment)</v>
       </c>
       <c r="AB26" t="str">
         <v/>
@@ -2923,7 +2937,7 @@
         <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized)</v>
       </c>
       <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated facility_utilization_status per facility.
+        <v xml:space="preserve">Calculated utilization_status_code per facility.
 </v>
       </c>
       <c r="E29" t="str">
@@ -2942,7 +2956,7 @@
         <v>Calc</v>
       </c>
       <c r="J29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated facility_utilization_status per facility.
+        <v xml:space="preserve">Calculated utilization_status_code per facility.
 </v>
       </c>
       <c r="K29" t="str">
@@ -2955,7 +2969,7 @@
         <v>Agg</v>
       </c>
       <c r="N29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level facility_utilization_status) per counterparty.
+        <v xml:space="preserve">SUM(facility-level utilization_status_code) per counterparty.
 </v>
       </c>
       <c r="O29" t="str">
@@ -2968,7 +2982,7 @@
         <v>Agg</v>
       </c>
       <c r="R29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_utilization_status per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level utilization_status_code per L3 desk segment.
 </v>
       </c>
       <c r="S29" t="str">
@@ -2981,7 +2995,7 @@
         <v>Agg</v>
       </c>
       <c r="V29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_utilization_status per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level utilization_status_code per L2 portfolio segment.
 </v>
       </c>
       <c r="W29" t="str">
@@ -2994,7 +3008,7 @@
         <v>Agg</v>
       </c>
       <c r="Z29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_utilization_status per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level utilization_status_code per L1 business segment segment.
 </v>
       </c>
       <c r="AA29" t="str">
@@ -4683,14 +4697,15 @@
         <v>EXP-041</v>
       </c>
       <c r="B48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Total interest earned on outstanding exposures during the reporting period.
+        <v xml:space="preserve">Total interest earned on outstanding exposures during the reporting period. Sources from facility_profitability_snapshot.interest_income_amt (ETL'd from core banking, includes proper accrual and day-count per ASC 310-20). Bank-share-adjusted via facility_lender_allocation.
 </v>
       </c>
       <c r="C48" t="str">
         <v>Interest Income</v>
       </c>
       <c r="D48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(interest_income_amt) per facility from facility_profitability_snapshot. Weighted by bank share percentage.
+        <v xml:space="preserve">SUM(interest_income_amt) per facility from facility_profitability_snapshot.
+Weighted by bank_share_pct from facility_lender_allocation.
 </v>
       </c>
       <c r="E48" t="str">
@@ -4709,7 +4724,8 @@
         <v>Agg</v>
       </c>
       <c r="J48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(interest_income_amt) per facility from facility_profitability_snapshot. Weighted by bank share percentage.
+        <v xml:space="preserve">SUM(interest_income_amt) per facility from facility_profitability_snapshot.
+Weighted by bank_share_pct from facility_lender_allocation.
 </v>
       </c>
       <c r="K48" t="str">
@@ -4719,10 +4735,11 @@
         <v>Y</v>
       </c>
       <c r="M48" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level interest_income_amt per counterparty.
+        <v xml:space="preserve">For each counterparty, sum facility-level interest income weighted
+by participation_pct from facility_counterparty_participation.
 </v>
       </c>
       <c r="O48" t="str">
@@ -4735,7 +4752,7 @@
         <v>Agg</v>
       </c>
       <c r="R48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level interest_income_amt per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level interest income per L3 desk segment.
 </v>
       </c>
       <c r="S48" t="str">
@@ -4748,7 +4765,8 @@
         <v>Agg</v>
       </c>
       <c r="V48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level interest_income_amt per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level interest income per L2 portfolio segment.
+Traverses L3 -&gt; L2 via parent_segment_id.
 </v>
       </c>
       <c r="W48" t="str">
@@ -4761,7 +4779,8 @@
         <v>Agg</v>
       </c>
       <c r="Z48" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level interest_income_amt per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level interest income per L1 business segment.
+Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA48" t="str">
@@ -5899,7 +5918,7 @@
         <v>Pricing Tier</v>
       </c>
       <c r="D61" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier from facility_pricing_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Read pricing_tier_code from facility_detail_snapshot for each facility as-of reporting date.
 </v>
       </c>
       <c r="E61" t="str">
@@ -5918,7 +5937,7 @@
         <v>Raw</v>
       </c>
       <c r="J61" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier from facility_pricing_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Read pricing_tier_code from facility_detail_snapshot for each facility as-of reporting date.
 </v>
       </c>
       <c r="K61" t="str">
@@ -5931,7 +5950,7 @@
         <v>Raw</v>
       </c>
       <c r="N61" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier per counterparty.
+        <v xml:space="preserve">Read pricing_tier_code per counterparty.
 </v>
       </c>
       <c r="O61" t="str">
@@ -5944,7 +5963,7 @@
         <v>Agg</v>
       </c>
       <c r="R61" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L3 desk segment.
 </v>
       </c>
       <c r="S61" t="str">
@@ -5957,7 +5976,7 @@
         <v>Agg</v>
       </c>
       <c r="V61" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L2 portfolio segment.
 </v>
       </c>
       <c r="W61" t="str">
@@ -5970,7 +5989,7 @@
         <v>Agg</v>
       </c>
       <c r="Z61" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L1 business segment segment.
 </v>
       </c>
       <c r="AA61" t="str">
@@ -6264,14 +6283,19 @@
         <v>PROF-108</v>
       </c>
       <c r="B65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Total interest cost incurred on funding sources attributable to the reporting unit during the period. At facility level, computed as the product of the committed amount, the bank's participation share, and the cost of funds rate. At higher rollup levels, aggregated as the sum of facility-level interest expense.
+        <v xml:space="preserve">Annualized interest cost on drawn/funded exposure. Computed as SUM(funded_amount) * bank_share_pct * cost_of_funds_pct at facility level. Uses funded basis (actual drawn amounts from position_detail) rather than committed basis, aligning with FR Y-9C Schedule HI Item 2.
 </v>
       </c>
       <c r="C65" t="str">
         <v>Interest Expense</v>
       </c>
-      <c r="D65" t="str">
-        <v>committed_facility_amt × bank_share_pct × cost_of_funds_rate</v>
+      <c r="D65" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each active facility:
+1. Join position -&gt; position_detail, SUM(funded_amount) per facility
+2. Multiply by bank_share_pct / 100 from facility_lender_allocation
+3. Multiply by COALESCE(cost_of_funds_pct, all_in_rate_pct - spread_bps/100) / 100
+   from facility_pricing_snapshot
+</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -6288,8 +6312,13 @@
       <c r="I65" t="str">
         <v>Calc</v>
       </c>
-      <c r="J65" t="str">
-        <v>committed_facility_amt × bank_share_pct × cost_of_funds_rate</v>
+      <c r="J65" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each active facility:
+1. Join position -&gt; position_detail, SUM(funded_amount) per facility
+2. Multiply by bank_share_pct / 100 from facility_lender_allocation
+3. Multiply by COALESCE(cost_of_funds_pct, all_in_rate_pct - spread_bps/100) / 100
+   from facility_pricing_snapshot
+</v>
       </c>
       <c r="K65" t="str">
         <v>Interest Expense (facility)</v>
@@ -6298,10 +6327,12 @@
         <v>Y</v>
       </c>
       <c r="M65" t="str">
-        <v>Agg</v>
-      </c>
-      <c r="N65" t="str">
-        <v>SUM(Facility Interest Expense) per counterparty</v>
+        <v>Calc</v>
+      </c>
+      <c r="N65" t="str" xml:space="preserve">
+        <v xml:space="preserve">For each counterparty, sum facility-level interest expense weighted
+by participation_pct from facility_counterparty_participation.
+</v>
       </c>
       <c r="O65" t="str">
         <v>Interest Expense (counterparty)</v>
@@ -6312,8 +6343,9 @@
       <c r="Q65" t="str">
         <v>Agg</v>
       </c>
-      <c r="R65" t="str">
-        <v>SUM(Facility Interest Expense) per L3 desk segment</v>
+      <c r="R65" t="str" xml:space="preserve">
+        <v xml:space="preserve">SUM of facility-level interest expense per L3 desk segment.
+</v>
       </c>
       <c r="S65" t="str">
         <v>Interest Expense (desk)</v>
@@ -6324,8 +6356,10 @@
       <c r="U65" t="str">
         <v>Agg</v>
       </c>
-      <c r="V65" t="str">
-        <v>SUM(Facility Interest Expense) per L2 portfolio segment</v>
+      <c r="V65" t="str" xml:space="preserve">
+        <v xml:space="preserve">SUM of facility-level interest expense per L2 portfolio segment.
+Traverses L3 -&gt; L2 via parent_segment_id.
+</v>
       </c>
       <c r="W65" t="str">
         <v>Interest Expense (portfolio)</v>
@@ -6336,8 +6370,10 @@
       <c r="Y65" t="str">
         <v>Agg</v>
       </c>
-      <c r="Z65" t="str">
-        <v>SUM(Facility Interest Expense) per L1 business segment (department)</v>
+      <c r="Z65" t="str" xml:space="preserve">
+        <v xml:space="preserve">SUM of facility-level interest expense per L1 business segment.
+Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
+</v>
       </c>
       <c r="AA65" t="str">
         <v>Interest Expense (business_segment)</v>
@@ -7567,7 +7603,7 @@
         <v>Active</v>
       </c>
       <c r="D79" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of active_flag from facility_master.
+        <v xml:space="preserve">Direct lookup of is_active_flag from facility_master.
 </v>
       </c>
       <c r="E79" t="str">
@@ -7586,7 +7622,7 @@
         <v>Raw</v>
       </c>
       <c r="J79" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of active_flag from facility_master.
+        <v xml:space="preserve">Direct lookup of is_active_flag from facility_master.
 </v>
       </c>
       <c r="K79" t="str">
@@ -7599,7 +7635,7 @@
         <v>Raw</v>
       </c>
       <c r="N79" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read active_flag per counterparty.
+        <v xml:space="preserve">Read is_active_flag per counterparty.
 </v>
       </c>
       <c r="O79" t="str">
@@ -7612,7 +7648,7 @@
         <v>Agg</v>
       </c>
       <c r="R79" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level active_flag per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level is_active_flag per L3 desk segment.
 </v>
       </c>
       <c r="S79" t="str">
@@ -7625,7 +7661,7 @@
         <v>Agg</v>
       </c>
       <c r="V79" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level active_flag per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level is_active_flag per L2 portfolio segment.
 </v>
       </c>
       <c r="W79" t="str">
@@ -7638,7 +7674,7 @@
         <v>Agg</v>
       </c>
       <c r="Z79" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level active_flag per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level is_active_flag per L1 business segment segment.
 </v>
       </c>
       <c r="AA79" t="str">
@@ -9334,7 +9370,7 @@
         <v>Facility Active Flag</v>
       </c>
       <c r="D98" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated facility_active_flag per facility.
+        <v xml:space="preserve">Calculated facility_is_active_flag per facility.
 </v>
       </c>
       <c r="E98" t="str">
@@ -9353,7 +9389,7 @@
         <v>Calc</v>
       </c>
       <c r="J98" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated facility_active_flag per facility.
+        <v xml:space="preserve">Calculated facility_is_active_flag per facility.
 </v>
       </c>
       <c r="K98" t="str">
@@ -9366,7 +9402,7 @@
         <v>Agg</v>
       </c>
       <c r="N98" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level facility_active_flag) per counterparty.
+        <v xml:space="preserve">SUM(facility-level facility_is_active_flag) per counterparty.
 </v>
       </c>
       <c r="O98" t="str">
@@ -9379,7 +9415,7 @@
         <v>Agg</v>
       </c>
       <c r="R98" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_active_flag per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level facility_is_active_flag per L3 desk segment.
 </v>
       </c>
       <c r="S98" t="str">
@@ -9392,7 +9428,7 @@
         <v>Agg</v>
       </c>
       <c r="V98" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_active_flag per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level facility_is_active_flag per L2 portfolio segment.
 </v>
       </c>
       <c r="W98" t="str">
@@ -9405,7 +9441,7 @@
         <v>Agg</v>
       </c>
       <c r="Z98" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_active_flag per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level facility_is_active_flag per L1 business segment segment.
 </v>
       </c>
       <c r="AA98" t="str">

</xml_diff>

<commit_message>
Fix metric calculators: PRINCIPAL filter, cost_of_funds scale, undrawn derivation
- Filter position_detail to detail_type='PRINCIPAL' only in Outstanding
  Exposure (EXP-018), Undrawn Exposure (EXP-017), and Interest Expense
  (PROF-108) calculators and YAML SQL formulas. INTEREST/FEE rows were
  inflating funded/unfunded sums by 2-5x.

- Fix cost_of_funds_pct stored as decimal (0.048) instead of percentage
  (4.8) in facility_pricing_snapshot. Interest Expense was ~104x too low.

- Rewrite Undrawn Exposure formula from SUM(unfunded_amount) to
  (committed_facility_amt - SUM(funded_amount)) to guarantee the identity
  Committed = Outstanding + Undrawn (FR Y-14Q Fields 24-25).

- Regenerate demo data for all 5 metrics with corrected formulas.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -2537,7 +2537,7 @@
         <v>EXP-017</v>
       </c>
       <c r="B25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Bank-share-adjusted unfunded commitment amount. Measures contingent funding risk by summing unfunded positions per facility, applying the bank's share percentage from facility_lender_allocation. Derived as Committed Exposure minus Outstanding Exposure.
+        <v xml:space="preserve">Bank-share-adjusted unfunded commitment amount. Derived as committed_facility_amt minus SUM(funded_amount) from PRINCIPAL positions, multiplied by bank_share_pct / 100. Ensures the identity: Committed Exposure = Outstanding Exposure + Undrawn Exposure. Maps to FR Y-14Q Field 24 minus Field 25.
 </v>
       </c>
       <c r="C25" t="str">
@@ -2545,9 +2545,10 @@
       </c>
       <c r="D25" t="str" xml:space="preserve">
         <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(unfunded_amount) across all positions for the facility
+1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
+2. Subtract from committed_facility_amt to get unfunded amount
 3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
 </v>
       </c>
       <c r="E25" t="str">
@@ -2567,9 +2568,10 @@
       </c>
       <c r="J25" t="str" xml:space="preserve">
         <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(unfunded_amount) across all positions for the facility
+1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
+2. Subtract from committed_facility_amt to get unfunded amount
 3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
 </v>
       </c>
       <c r="K25" t="str">

</xml_diff>

<commit_message>
Move Average Tenor metric from deal_pipeline_fact to facility_master dates
Average Tenor (Years) now calculates from facility_master.maturity_date
and origination_date instead of deal_pipeline_fact.expected_tenor_months.
At facility level: (maturity_date - origination_date) / 365.25.
At higher levels: AVG across underlying facilities.

- Drop l3.deal_pipeline_calc table (PostgreSQL + DDL + l3-tables.ts)
- Rewrite REF-003 YAML: source_tables, formulas, all 5 rollup levels
- Update MET-007 catalogue: ingredient_fields, unit_type, viz config
- Regenerate catalogue + visualization configs via calc:sync

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -6575,14 +6575,14 @@
         <v>REF-003</v>
       </c>
       <c r="B68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Average tenor of the underlying facilities across exposures. For facility, displayed the calculated tenor based on Origination Date ("Effective Date") and Maturity Date ("End Date") and other levels this metric is aggregated as an average to represent the average period of the underlying facilities.
+        <v xml:space="preserve">Average tenor of the underlying facilities across exposures. For facility, displayed the calculated tenor based on Origination Date ("Effective Date") and Maturity Date ("End Date"). At other levels this metric is aggregated as an average to represent the average period of the underlying facilities. Calculated from l2.facility_master.maturity_date and origination_date.
 </v>
       </c>
       <c r="C68" t="str">
         <v>Average Tenor (Years)</v>
       </c>
       <c r="D68" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID, [Contract Level Maturity Date]- [Facility Level Effective Date]
+        <v xml:space="preserve">For each Facility_ID, (Maturity Date - Origination Date) / 365.25 to get tenor in years.
 </v>
       </c>
       <c r="E68" t="str">
@@ -6601,7 +6601,7 @@
         <v>Calc</v>
       </c>
       <c r="J68" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID, [Contract Level Maturity Date]- [Facility Level Effective Date]
+        <v xml:space="preserve">For each Facility_ID, (Maturity Date - Origination Date) / 365.25 to get tenor in years.
 </v>
       </c>
       <c r="K68" t="str">
@@ -6614,7 +6614,7 @@
         <v>Avg</v>
       </c>
       <c r="N68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of expected_tenor_months across counterparty facilities.
+        <v xml:space="preserve">Average of facility-level tenor (years) across counterparty facilities.
 </v>
       </c>
       <c r="O68" t="str">
@@ -6627,7 +6627,7 @@
         <v>Avg</v>
       </c>
       <c r="R68" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level expected_tenor_months per L3 desk segment.
+        <v xml:space="preserve">AVG of facility-level tenor (years) per L3 desk segment.
 </v>
       </c>
       <c r="S68" t="str">
@@ -6640,7 +6640,7 @@
         <v>Avg</v>
       </c>
       <c r="V68" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level expected_tenor_months per L2 portfolio segment.
+        <v xml:space="preserve">AVG of facility-level tenor (years) per L2 portfolio segment.
 </v>
       </c>
       <c r="W68" t="str">
@@ -6650,10 +6650,10 @@
         <v>Y</v>
       </c>
       <c r="Y68" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="Z68" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_tenor_months per L1 business segment segment.
+        <v xml:space="preserve">AVG of facility-level tenor (years) per L1 business segment.
 </v>
       </c>
       <c r="AA68" t="str">

</xml_diff>

<commit_message>
GSIB audit remediation: FK constraints, descriptions, regulatory tables, YAML fixes
8-phase remediation addressing 30+ CRITICAL audit findings:

Phase 0: Backfill 1769 field descriptions, governance metadata, deprecated annotations
Phase 1: Create 9 missing L3 overlay tables (facility_exposure_calc, etc.)
Phase 2: Annotate L2/L3 convention violations in data dictionary
Phase 3: Fix 7 YAML metric definitions (CAP-001/002, RSK-001, AMD-001, EXP-009/045/046)
Phase 4: Add audit fields (record_source, load_timestamp, etc.) to all tables
Phase 5: Add currency_code to 13 L2 tables with monetary amounts
Phase 6: Generate and apply 195 FK constraints (55 L1 + 139 L2 + 1 L3)
Phase 7: Add 10 regulatory coverage tables (ECL/CECL, Watchlist, Forbearance)

Key results: 0→195 FK constraints, 32%→95%+ field descriptions, 0→499 relationships,
7 broken YAML metrics fixed, 10 new regulatory tables, full governance metadata.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1828,7 +1828,7 @@
         <v>Agg</v>
       </c>
       <c r="N17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per counterparty.
+        <v xml:space="preserve">MAX (worst bucket) of facility-level dpd_bucket_code per counterparty.
 </v>
       </c>
       <c r="O17" t="str">
@@ -1841,7 +1841,7 @@
         <v>Agg</v>
       </c>
       <c r="R17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L3 desk segment.
+        <v xml:space="preserve">MAX (worst bucket) of facility-level dpd_bucket_code per L3 desk segment.
 </v>
       </c>
       <c r="S17" t="str">
@@ -1854,7 +1854,7 @@
         <v>Agg</v>
       </c>
       <c r="V17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L2 portfolio segment.
+        <v xml:space="preserve">MAX (worst bucket) of facility-level dpd_bucket_code per L2 portfolio segment.
 </v>
       </c>
       <c r="W17" t="str">
@@ -1867,7 +1867,7 @@
         <v>Agg</v>
       </c>
       <c r="Z17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L1 business segment segment.
+        <v xml:space="preserve">MAX (worst bucket) of facility-level dpd_bucket_code per L1 business segment.
 </v>
       </c>
       <c r="AA17" t="str">
@@ -5205,10 +5205,10 @@
         <v>Y</v>
       </c>
       <c r="M53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="N53" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of rwa_amt across counterparty facilities.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per counterparty.
 </v>
       </c>
       <c r="O53" t="str">
@@ -5231,10 +5231,10 @@
         <v>Y</v>
       </c>
       <c r="U53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="V53" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level rwa_amt per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per L2 portfolio segment.
 </v>
       </c>
       <c r="W53" t="str">
@@ -5244,10 +5244,10 @@
         <v>Y</v>
       </c>
       <c r="Y53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="Z53" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level rwa_amt per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per L1 business segment.
 </v>
       </c>
       <c r="AA53" t="str">

</xml_diff>

<commit_message>
Fix audit findings: 5 metric formula bugs, 2 UNIQUE constraints, 3 layer fixes
Phase 1 — Metric YAML formula fixes:
- RSK-001: Fix hardcoded `1 AS metric_value` → `cro.rating_grade_id`
- EXP-009: Change SUM→MAX on VARCHAR dpd_bucket_code at all rollup levels
- EXP-001: Remove bank_share_pct from GROUP BY (prevents duplicate rows)
- CAP-001/CAP-002: Add missing LEFT JOIN to facility_exposure_calc with COALESCE fallback

Phase 1 — Structural integrity:
- Migration 005: Add UNIQUE constraints on facility_exposure_snapshot and counterparty_rating_observation

Phase 2 — Layer consistency:
- Remove metric_threshold from l1-table-meta.ts (belongs in L2)
- Rename L3 stress_test_result → facility_stress_test_calc (resolves L2/L3 name collision)
- Fix EXP-016: update table ref + field name (expected_loss_usd → stressed_expected_loss)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1828,7 +1828,7 @@
         <v>Agg</v>
       </c>
       <c r="N17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per counterparty.
+        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per counterparty.
 </v>
       </c>
       <c r="O17" t="str">
@@ -1841,7 +1841,7 @@
         <v>Agg</v>
       </c>
       <c r="R17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L3 desk segment.
+        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L3 desk segment.
 </v>
       </c>
       <c r="S17" t="str">
@@ -1854,7 +1854,7 @@
         <v>Agg</v>
       </c>
       <c r="V17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L2 portfolio segment.
+        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L2 portfolio segment.
 </v>
       </c>
       <c r="W17" t="str">
@@ -1867,7 +1867,7 @@
         <v>Agg</v>
       </c>
       <c r="Z17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level dpd_bucket_code per L1 business segment segment.
+        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L1 business segment.
 </v>
       </c>
       <c r="AA17" t="str">
@@ -2451,7 +2451,7 @@
         <v>Expected Loss ($)</v>
       </c>
       <c r="D24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(expected_loss_usd) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
 </v>
       </c>
       <c r="E24" t="str">
@@ -2470,7 +2470,7 @@
         <v>Agg</v>
       </c>
       <c r="J24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(expected_loss_usd) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
 </v>
       </c>
       <c r="K24" t="str">
@@ -2483,7 +2483,7 @@
         <v>Agg</v>
       </c>
       <c r="N24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_usd per counterparty.
+        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per counterparty.
 </v>
       </c>
       <c r="O24" t="str">
@@ -2496,7 +2496,7 @@
         <v>Agg</v>
       </c>
       <c r="R24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_usd per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L3 desk segment.
 </v>
       </c>
       <c r="S24" t="str">
@@ -2509,7 +2509,7 @@
         <v>Agg</v>
       </c>
       <c r="V24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_usd per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L2 portfolio segment.
 </v>
       </c>
       <c r="W24" t="str">
@@ -2522,7 +2522,7 @@
         <v>Agg</v>
       </c>
       <c r="Z24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_usd per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L1 business segment segment.
 </v>
       </c>
       <c r="AA24" t="str">

</xml_diff>

<commit_message>
GSIB audit remediation: BCBS 239 fields, catalogue sync, validation fixes
- Add SCD-2 temporal fields to 33 remaining L1 tables (migration 016)
- Add run_id/model_version lineage to 75 L3 tables (migration 017)
- Add record_source to 6 L1/L2 tables (migration 018)
- Sync metric catalogue from 5→105 items via YAML pipeline
- Fix DDL flag renames (is_default_flag, is_result_flag, etc.)
- Remove phantom revenue_amt from facility_financial_calc DDL
- Update validator: supplementary DDL, domain-prefixed metrics, allowlist
- Introspect DB: 254 new fields, 5 dashboard derived tables deployed
- Final validation: 26 PASS / 10 WARN / 0 FAIL

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -5205,10 +5205,10 @@
         <v>Y</v>
       </c>
       <c r="M53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="N53" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of rwa_amt across counterparty facilities.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per counterparty.
 </v>
       </c>
       <c r="O53" t="str">
@@ -5231,10 +5231,10 @@
         <v>Y</v>
       </c>
       <c r="U53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="V53" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level rwa_amt per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per L2 portfolio segment.
 </v>
       </c>
       <c r="W53" t="str">
@@ -5244,10 +5244,10 @@
         <v>Y</v>
       </c>
       <c r="Y53" t="str">
-        <v>Avg</v>
+        <v>Agg</v>
       </c>
       <c r="Z53" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level rwa_amt per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level rwa_amt per L1 business segment.
 </v>
       </c>
       <c r="AA53" t="str">

</xml_diff>

<commit_message>
Metric library v2: 5 GSIB metrics with DB-validated rollup formulas
- REF-001 (NOL): Fix source table L3→L2, COALESCE(0) at all levels
- AMD-001 (ASD): Rewrite to MAX(effective_date) from amendment_event
- AMD-002 (ASC): Rewrite to COUNT by status category with dim lookup
- AMD-003 (ATC): Rewrite to COUNT by type category with dim lookup
- EXP-014 (DSCR): Rewrite to sum-ratio from L2 NOI/debt service ingredients
- Enhance sync-yaml-to-catalogue to propagate status, abbreviation, name,
  definition, metric_class, direction, domain, insight, regulatory refs
- Set 5 reviewed metrics ACTIVE, others DRAFT; UI filters by status
- All formulas tested against PostgreSQL with consistent rollups at all 5
  hierarchy levels (facility→counterparty→desk→portfolio→segment)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -487,14 +487,19 @@
         <v>AMD-001</v>
       </c>
       <c r="B3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Date amendment became effective.
+        <v xml:space="preserve">Effective date of the most recent amendment on a facility. At rollup levels,
+reports the latest (MAX) amendment effective date across the group — shows
+how recently amendment activity occurred within each counterparty, desk,
+portfolio, or business segment.
 </v>
       </c>
       <c r="C3" t="str">
         <v>Amendment Start Date</v>
       </c>
       <c r="D3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read effective_date from facility_master for each facility.
+        <v xml:space="preserve">Latest amendment effective_date per facility, converted to epoch seconds
+for numeric comparison. One facility may have multiple amendments;
+MAX selects the most recent.
 </v>
       </c>
       <c r="E3" t="str">
@@ -513,7 +518,9 @@
         <v>Raw</v>
       </c>
       <c r="J3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read effective_date from facility_master for each facility.
+        <v xml:space="preserve">Latest amendment effective_date per facility, converted to epoch seconds
+for numeric comparison. One facility may have multiple amendments;
+MAX selects the most recent.
 </v>
       </c>
       <c r="K3" t="str">
@@ -526,7 +533,8 @@
         <v>Agg</v>
       </c>
       <c r="N3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Latest (MAX) effective_date per counterparty.
+        <v xml:space="preserve">Latest amendment effective_date across all facilities for each
+counterparty. Uses amendment_event.counterparty_id directly.
 </v>
       </c>
       <c r="O3" t="str">
@@ -539,7 +547,7 @@
         <v>Agg</v>
       </c>
       <c r="R3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Latest (MAX) effective_date per L3 desk segment.
+        <v xml:space="preserve">Latest amendment effective_date per L3 desk segment.
 </v>
       </c>
       <c r="S3" t="str">
@@ -552,7 +560,8 @@
         <v>Agg</v>
       </c>
       <c r="V3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Latest (MAX) effective_date per L2 portfolio segment.
+        <v xml:space="preserve">Latest amendment effective_date per L2 portfolio segment.
+Walks up hierarchy: L3 desk → L2 portfolio via parent_segment_id.
 </v>
       </c>
       <c r="W3" t="str">
@@ -565,7 +574,8 @@
         <v>Agg</v>
       </c>
       <c r="Z3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Latest (MAX) effective_date per L1 business segment.
+        <v xml:space="preserve">Latest amendment effective_date per L1 business segment.
+Walks up hierarchy: L3 → L2 → L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA3" t="str">
@@ -580,14 +590,19 @@
         <v>AMD-002</v>
       </c>
       <c r="B4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Status of amendment within the approval lifecycle.
+        <v xml:space="preserve">Count of amendments by approval lifecycle status (e.g., Prospect Identified,
+In Underwriting, Under Credit Review, Pending Approval, Complete, Rejected).
+At each rollup level, provides a distribution breakdown showing how many
+amendments fall into each status category. Key CRO indicator for amendment
+pipeline health and bottleneck identification.
 </v>
       </c>
       <c r="C4" t="str">
-        <v>Amendment Status</v>
+        <v>Amendment Status Count</v>
       </c>
       <c r="D4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read amendment status flag for each active facility.
+        <v xml:space="preserve">Count of amendments per facility, broken out by status category.
+Each row represents one (facility, status) combination with its count.
 </v>
       </c>
       <c r="E4" t="str">
@@ -606,11 +621,12 @@
         <v>Raw</v>
       </c>
       <c r="J4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read amendment status flag for each active facility.
+        <v xml:space="preserve">Count of amendments per facility, broken out by status category.
+Each row represents one (facility, status) combination with its count.
 </v>
       </c>
       <c r="K4" t="str">
-        <v>Amendment Status (facility)</v>
+        <v>Amendment Status Count (facility)</v>
       </c>
       <c r="L4" t="str">
         <v>Y</v>
@@ -619,11 +635,13 @@
         <v>Agg</v>
       </c>
       <c r="N4" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with amendment status per counterparty.
+        <v xml:space="preserve">Count of amendments per counterparty by status category.
+Uses amendment_event.counterparty_id directly (no participation weighting —
+amendments are discrete events, not divisible by ownership share).
 </v>
       </c>
       <c r="O4" t="str">
-        <v>Amendment Status (counterparty)</v>
+        <v>Amendment Status Count (counterparty)</v>
       </c>
       <c r="P4" t="str">
         <v>Y</v>
@@ -632,11 +650,11 @@
         <v>Agg</v>
       </c>
       <c r="R4" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with amendment status per L3 desk segment.
+        <v xml:space="preserve">Count of amendments per L3 desk segment by status category.
 </v>
       </c>
       <c r="S4" t="str">
-        <v>Amendment Status (desk)</v>
+        <v>Amendment Status Count (desk)</v>
       </c>
       <c r="T4" t="str">
         <v>Y</v>
@@ -645,11 +663,12 @@
         <v>Agg</v>
       </c>
       <c r="V4" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with amendment status per L2 portfolio segment.
+        <v xml:space="preserve">Count of amendments per L2 portfolio segment by status category.
+Walks up hierarchy: L3 desk → L2 portfolio via parent_segment_id.
 </v>
       </c>
       <c r="W4" t="str">
-        <v>Amendment Status (portfolio)</v>
+        <v>Amendment Status Count (portfolio)</v>
       </c>
       <c r="X4" t="str">
         <v>Y</v>
@@ -658,11 +677,12 @@
         <v>Agg</v>
       </c>
       <c r="Z4" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with amendment status per L1 business segment.
+        <v xml:space="preserve">Count of amendments per L1 business segment by status category.
+Walks up hierarchy: L3 → L2 → L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA4" t="str">
-        <v>Amendment Status (business_segment)</v>
+        <v>Amendment Status Count (business_segment)</v>
       </c>
       <c r="AB4" t="str">
         <v/>
@@ -673,14 +693,18 @@
         <v>AMD-003</v>
       </c>
       <c r="B5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Type of contractual amendment (e.g., covenant reset, maturity extension).
+        <v xml:space="preserve">Count of amendments by contractual type (e.g., Commitment Changes, Pricing,
+Tenor-Maturity, Amortization, Currency). At each rollup level, provides a
+distribution breakdown showing amendment activity by type category.
+Key CRO indicator for understanding what credit terms are being renegotiated.
 </v>
       </c>
       <c r="C5" t="str">
-        <v>Amendment Type</v>
+        <v>Amendment Type Count</v>
       </c>
       <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of amendment_type_code from amendment_type_dim.
+        <v xml:space="preserve">Count of amendments per facility, broken out by amendment type.
+Each row represents one (facility, type) combination with its count.
 </v>
       </c>
       <c r="E5" t="str">
@@ -699,11 +723,12 @@
         <v>Raw</v>
       </c>
       <c r="J5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of amendment_type_code from amendment_type_dim.
+        <v xml:space="preserve">Count of amendments per facility, broken out by amendment type.
+Each row represents one (facility, type) combination with its count.
 </v>
       </c>
       <c r="K5" t="str">
-        <v>Amendment Type (facility)</v>
+        <v>Amendment Type Count (facility)</v>
       </c>
       <c r="L5" t="str">
         <v>Y</v>
@@ -712,11 +737,13 @@
         <v>Agg</v>
       </c>
       <c r="N5" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level amendment_type_code) per counterparty.
+        <v xml:space="preserve">Count of amendments per counterparty by type category.
+Uses amendment_event.counterparty_id directly (amendments are
+discrete events, not weighted by participation share).
 </v>
       </c>
       <c r="O5" t="str">
-        <v>Amendment Type (counterparty)</v>
+        <v>Amendment Type Count (counterparty)</v>
       </c>
       <c r="P5" t="str">
         <v>Y</v>
@@ -725,11 +752,11 @@
         <v>Agg</v>
       </c>
       <c r="R5" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level amendment_type_code per L3 desk segment.
+        <v xml:space="preserve">Count of amendments per L3 desk segment by type category.
 </v>
       </c>
       <c r="S5" t="str">
-        <v>Amendment Type (desk)</v>
+        <v>Amendment Type Count (desk)</v>
       </c>
       <c r="T5" t="str">
         <v>Y</v>
@@ -738,11 +765,12 @@
         <v>Agg</v>
       </c>
       <c r="V5" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level amendment_type_code per L2 portfolio segment.
+        <v xml:space="preserve">Count of amendments per L2 portfolio segment by type category.
+Walks up hierarchy: L3 desk → L2 portfolio via parent_segment_id.
 </v>
       </c>
       <c r="W5" t="str">
-        <v>Amendment Type (portfolio)</v>
+        <v>Amendment Type Count (portfolio)</v>
       </c>
       <c r="X5" t="str">
         <v>Y</v>
@@ -751,11 +779,12 @@
         <v>Agg</v>
       </c>
       <c r="Z5" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level amendment_type_code per L1 business segment segment.
+        <v xml:space="preserve">Count of amendments per L1 business segment by type category.
+Walks up hierarchy: L3 → L2 → L1 via parent_segment_id chain.
 </v>
       </c>
       <c r="AA5" t="str">
-        <v>Amendment Type (business_segment)</v>
+        <v>Amendment Type Count (business_segment)</v>
       </c>
       <c r="AB5" t="str">
         <v/>
@@ -2254,14 +2283,26 @@
         <v>EXP-014</v>
       </c>
       <c r="B22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Net Operating Income divided by Total Debt Service. Measures borrower's ability to meet debt obligations from operating cash flow, providing insight into covenant compliance and credit resilience.
+        <v xml:space="preserve">Cashflow (Net Operating Income) divided by Total Debt Service (Interest Expense + Principal Payments). Measures borrower's ability to meet debt obligations from operating cash flow. DSCR &gt; 1.0 means the borrower generates enough income to cover debt payments. Key covenant compliance and credit resilience indicator.
+Ingredient derivation:
+  - NOI (noi_amt): L2 facility_financial_snapshot — raw atomic input
+  - Interest Expense (interest_expense_amt): L2 facility_financial_snapshot — raw
+  - Principal Payment (principal_payment_amt): L2 facility_financial_snapshot — raw
+  - Total Debt Service = interest_expense_amt + principal_payment_amt (L3 derived)
+  - DSCR = noi_amt / Total Debt Service (L3 derived)
+Rollup uses sum-ratio pattern: SUM(NOI) / SUM(Debt Service) at each level, preserving the mathematical relationship between numerator and denominator.
 </v>
       </c>
       <c r="C22" t="str">
         <v>Debt Service Coverage Ratio (DSCR)</v>
       </c>
       <c r="D22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Compute DSCR = noi_amt / total_debt_service_amt per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD noi_amt, interest_expense_amt, principal_payment_amt
+     from l2.facility_financial_snapshot
+  2. COMPUTE Total Debt Service = interest_expense_amt + principal_payment_amt
+  3. COMPUTE DSCR = noi_amt / Total Debt Service
+Ingredients: noi_amt (L2), interest_expense_amt (L2), principal_payment_amt (L2)
 </v>
       </c>
       <c r="E22" t="str">
@@ -2280,7 +2321,12 @@
         <v>Raw</v>
       </c>
       <c r="J22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Compute DSCR = noi_amt / total_debt_service_amt per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD noi_amt, interest_expense_amt, principal_payment_amt
+     from l2.facility_financial_snapshot
+  2. COMPUTE Total Debt Service = interest_expense_amt + principal_payment_amt
+  3. COMPUTE DSCR = noi_amt / Total Debt Service
+Ingredients: noi_amt (L2), interest_expense_amt (L2), principal_payment_amt (L2)
 </v>
       </c>
       <c r="K22" t="str">
@@ -2293,8 +2339,13 @@
         <v>Calc</v>
       </c>
       <c r="N22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average DSCR per counterparty:
-SUM(dscr * drawn_amount) / SUM(drawn_amount).
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD all facility-level ingredients (noi_amt, interest_expense_amt,
+     principal_payment_amt) for facilities belonging to this counterparty
+  2. COMPUTE SUM(noi_amt) across all facilities = Counterparty Cashflow
+  3. COMPUTE SUM(interest_expense_amt + principal_payment_amt) = Counterparty Debt Service
+  4. COMPUTE Counterparty DSCR = Counterparty Cashflow / Counterparty Debt Service
+Sum-ratio rollup preserves ingredient traceability.
 </v>
       </c>
       <c r="O22" t="str">
@@ -2307,8 +2358,12 @@
         <v>Calc</v>
       </c>
       <c r="R22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average DSCR per L3 desk segment:
-SUM(dscr * drawn_amount) / SUM(drawn_amount).
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+     via facility_master.lob_segment_id
+  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+     for all facilities mapped to this desk
+Sum-ratio rollup: aggregate ingredients first, then divide.
 </v>
       </c>
       <c r="S22" t="str">
@@ -2321,8 +2376,11 @@
         <v>Calc</v>
       </c>
       <c r="V22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average DSCR per L2 portfolio segment:
-SUM(dscr * drawn_amount) / SUM(drawn_amount).
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+     for all facilities whose desk rolls up to this portfolio
+Sum-ratio rollup: aggregate ingredients first, then divide.
 </v>
       </c>
       <c r="W22" t="str">
@@ -2335,8 +2393,11 @@
         <v>Calc</v>
       </c>
       <c r="Z22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average DSCR per L1 business segment:
-SUM(dscr * drawn_amount) / SUM(drawn_amount).
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+     for all facilities whose desk ultimately rolls up to this segment
+Sum-ratio rollup: aggregate ingredients first, then divide.
 </v>
       </c>
       <c r="AA22" t="str">

</xml_diff>

<commit_message>
Align 5 GSIB metrics to rollup spec with DB-validated formulas
MET-001: COUNT DISTINCT from l2.position, materialize to L3, SUM at higher levels
MET-002: Bank-share weighted avg (committed_amount * bank_share_pct), Calc at portfolio/LoB
MET-003: in_record=false for desk/portfolio/lob (dates don't aggregate at org levels)
MET-004: Categorical COUNT by amendment status at all 5 levels
MET-005: Categorical COUNT by amendment type, counterparty in_record=false per spec

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -5548,7 +5548,7 @@
         <v>Avg</v>
       </c>
       <c r="N56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average all_in_rate_pct per counterparty.
+        <v xml:space="preserve">For each Counterparty_ID, lookup Facility_IDs in Facility Master where IS(Counterparty_ID), SELECT all_in_rate_pct. Weight by bank share committed amount (committed_amount * bank_share_pct). Weighted average = SUM(rate * weight) / SUM(weight).
 </v>
       </c>
       <c r="O56" t="str">
@@ -5561,7 +5561,7 @@
         <v>Avg</v>
       </c>
       <c r="R56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average all_in_rate_pct per L3 desk segment.
+        <v xml:space="preserve">For each L3 LoB, lookup lob_segment_id from enterprise_business_taxonomy, then lookup facility_id in Facility Master where IS(lob_segment_id). SELECT all_in_rate_pct, weight by bank share committed exposure (committed_amount * bank_share_pct). Weighted average = SUM(rate * weight) / SUM(weight).
 </v>
       </c>
       <c r="S56" t="str">
@@ -5571,10 +5571,10 @@
         <v>Y</v>
       </c>
       <c r="U56" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="V56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average all_in_rate_pct per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 LoB, lookup lob_segment_id from enterprise_business_taxonomy, then lookup facility_id in Facility Master where IS(lob_segment_id). SELECT all_in_rate_pct, weight by bank share committed exposure (committed_amount * bank_share_pct). Calculated = SUM(rate * weight) / SUM(weight).
 </v>
       </c>
       <c r="W56" t="str">
@@ -5584,10 +5584,10 @@
         <v>Y</v>
       </c>
       <c r="Y56" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="Z56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average all_in_rate_pct per L1 business segment.
+        <v xml:space="preserve">For each L1 LoB, lookup lob_segment_id from enterprise_business_taxonomy, then lookup facility_id in Facility Master where IS(lob_segment_id). SELECT all_in_rate_pct, weight by bank share committed exposure (committed_amount * bank_share_pct). Calculated = SUM(rate * weight) / SUM(weight).
 </v>
       </c>
       <c r="AA56" t="str">
@@ -6457,7 +6457,7 @@
         <v>Number of Loans</v>
       </c>
       <c r="D66" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read number_of_loans from facility_exposure_snapshot for each facility.
+        <v xml:space="preserve">For each Facility_ID, COUNT DISTINCT(Position_ID) from l2.position. Result materialized to l3.facility_exposure_calc.number_of_loans.
 </v>
       </c>
       <c r="E66" t="str">
@@ -6473,10 +6473,10 @@
         <v>Y</v>
       </c>
       <c r="I66" t="str">
-        <v>Raw</v>
+        <v>Agg</v>
       </c>
       <c r="J66" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read number_of_loans from facility_exposure_snapshot for each facility.
+        <v xml:space="preserve">For each Facility_ID, COUNT DISTINCT(Position_ID) from l2.position. Result materialized to l3.facility_exposure_calc.number_of_loans.
 </v>
       </c>
       <c r="K66" t="str">
@@ -6489,7 +6489,7 @@
         <v>Agg</v>
       </c>
       <c r="N66" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of number_of_loans per counterparty.
+        <v xml:space="preserve">For each Counterparty_ID, lookup in Facility Table when IS(Counterparty_ID), SUM(Number_of_loans) from l3.facility_exposure_calc.
 </v>
       </c>
       <c r="O66" t="str">
@@ -6502,7 +6502,7 @@
         <v>Agg</v>
       </c>
       <c r="R66" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of number_of_loans per L3 desk segment.
+        <v xml:space="preserve">For each L3 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L3', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
 </v>
       </c>
       <c r="S66" t="str">
@@ -6515,7 +6515,7 @@
         <v>Agg</v>
       </c>
       <c r="V66" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of number_of_loans per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L2', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
 </v>
       </c>
       <c r="W66" t="str">
@@ -6528,7 +6528,7 @@
         <v>Agg</v>
       </c>
       <c r="Z66" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of number_of_loans per L1 business segment.
+        <v xml:space="preserve">For each L1 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L1', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
 </v>
       </c>
       <c r="AA66" t="str">

</xml_diff>

<commit_message>
Add FX currency conversion to DSCR, TDS, and FCCR aggregate formulas
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -2342,10 +2342,11 @@
         <v xml:space="preserve">For each counterparty:
   1. LOAD all facility-level ingredients (noi_amt, interest_expense_amt,
      principal_payment_amt) for facilities belonging to this counterparty
-  2. COMPUTE SUM(noi_amt) across all facilities = Counterparty Cashflow
-  3. COMPUTE SUM(interest_expense_amt + principal_payment_amt) = Counterparty Debt Service
-  4. COMPUTE Counterparty DSCR = Counterparty Cashflow / Counterparty Debt Service
-Sum-ratio rollup preserves ingredient traceability.
+  2. CONVERT amounts to USD via l2.fx_rate spot rate (COALESCE to 1 for USD-denominated)
+  3. COMPUTE SUM(noi_amt × fx_rate) across all facilities = Counterparty Cashflow (USD)
+  4. COMPUTE SUM((interest_expense + principal_payment) × fx_rate) = Counterparty Debt Service (USD)
+  5. COMPUTE Counterparty DSCR = Counterparty Cashflow / Counterparty Debt Service
+Sum-ratio rollup with FX conversion preserves ingredient traceability across currencies.
 </v>
       </c>
       <c r="O22" t="str">
@@ -2361,9 +2362,10 @@
         <v xml:space="preserve">For each L3 Desk segment:
   1. LOOKUP managed_segment_id from enterprise_business_taxonomy
      via facility_master.lob_segment_id
-  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+  2. CONVERT amounts to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(noi_amt × fx_rate) / SUM((interest_expense + principal_payment) × fx_rate)
      for all facilities mapped to this desk
-Sum-ratio rollup: aggregate ingredients first, then divide.
+Sum-ratio rollup with FX conversion: aggregate USD-converted ingredients first, then divide.
 </v>
       </c>
       <c r="S22" t="str">
@@ -2378,9 +2380,10 @@
       <c r="V22" t="str" xml:space="preserve">
         <v xml:space="preserve">For each L2 Portfolio segment:
   1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
-  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+  2. CONVERT amounts to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(noi_amt × fx_rate) / SUM((interest_expense + principal_payment) × fx_rate)
      for all facilities whose desk rolls up to this portfolio
-Sum-ratio rollup: aggregate ingredients first, then divide.
+Sum-ratio rollup with FX conversion: aggregate USD-converted ingredients first, then divide.
 </v>
       </c>
       <c r="W22" t="str">
@@ -2395,9 +2398,10 @@
       <c r="Z22" t="str" xml:space="preserve">
         <v xml:space="preserve">For each L1 Business Segment / LoB:
   1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
-  2. COMPUTE SUM(noi_amt) / SUM(interest_expense + principal_payment)
+  2. CONVERT amounts to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(noi_amt × fx_rate) / SUM((interest_expense + principal_payment) × fx_rate)
      for all facilities whose desk ultimately rolls up to this segment
-Sum-ratio rollup: aggregate ingredients first, then divide.
+Sum-ratio rollup with FX conversion: aggregate USD-converted ingredients first, then divide.
 </v>
       </c>
       <c r="AA22" t="str">
@@ -4488,7 +4492,7 @@
         <v>Total Debt Service ($)</v>
       </c>
       <c r="D45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup Position_ID for each Facility_ID, Select bank_share and cost_of_funds from Facility_ID from Facility Master THEN (unfunded_amt * bank_share ) = [Facility Debt Service w/ Bank Share]
+        <v xml:space="preserve">Lookup total_debt_service_amt from facility_financial_snapshot, convert to USD via l2.fx_rate spot rate (COALESCE to 1 for USD-denominated facilities).
 </v>
       </c>
       <c r="E45" t="str">
@@ -4507,7 +4511,7 @@
         <v>Calc</v>
       </c>
       <c r="J45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup Position_ID for each Facility_ID, Select bank_share and cost_of_funds from Facility_ID from Facility Master THEN (unfunded_amt * bank_share ) = [Facility Debt Service w/ Bank Share]
+        <v xml:space="preserve">Lookup total_debt_service_amt from facility_financial_snapshot, convert to USD via l2.fx_rate spot rate (COALESCE to 1 for USD-denominated facilities).
 </v>
       </c>
       <c r="K45" t="str">
@@ -4520,7 +4524,7 @@
         <v>Agg</v>
       </c>
       <c r="N45" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_debt_service_amt per counterparty.
+        <v xml:space="preserve">SUM of facility-level total_debt_service_amt converted to USD per counterparty.
 </v>
       </c>
       <c r="O45" t="str">
@@ -4533,7 +4537,7 @@
         <v>Agg</v>
       </c>
       <c r="R45" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_debt_service_amt per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level total_debt_service_amt converted to USD per L3 desk segment.
 </v>
       </c>
       <c r="S45" t="str">
@@ -4546,7 +4550,7 @@
         <v>Agg</v>
       </c>
       <c r="V45" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_debt_service_amt per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level total_debt_service_amt converted to USD per L2 portfolio segment.
 </v>
       </c>
       <c r="W45" t="str">
@@ -4559,7 +4563,7 @@
         <v>Agg</v>
       </c>
       <c r="Z45" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_debt_service_amt per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level total_debt_service_amt converted to USD per L1 business segment.
 </v>
       </c>
       <c r="AA45" t="str">
@@ -5362,7 +5366,8 @@
         <v>Calc</v>
       </c>
       <c r="N54" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(ebitda) / SUM(total_debt_service) per counterparty.
+        <v xml:space="preserve">SUM(ebitda × fx_rate) / SUM(total_debt_service × fx_rate) per counterparty.
+Amounts converted to USD via l2.fx_rate before aggregation.
 </v>
       </c>
       <c r="O54" t="str">
@@ -5375,7 +5380,8 @@
         <v>Calc</v>
       </c>
       <c r="R54" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(ebitda) / SUM(total_debt_service) per L3 desk segment.
+        <v xml:space="preserve">SUM(ebitda × fx_rate) / SUM(total_debt_service × fx_rate) per L3 desk segment.
+Amounts converted to USD via l2.fx_rate before aggregation.
 </v>
       </c>
       <c r="S54" t="str">
@@ -5388,7 +5394,8 @@
         <v>Calc</v>
       </c>
       <c r="V54" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(ebitda) / SUM(total_debt_service) per L2 portfolio segment.
+        <v xml:space="preserve">SUM(ebitda × fx_rate) / SUM(total_debt_service × fx_rate) per L2 portfolio segment.
+Amounts converted to USD via l2.fx_rate before aggregation.
 </v>
       </c>
       <c r="W54" t="str">
@@ -5401,7 +5408,8 @@
         <v>Calc</v>
       </c>
       <c r="Z54" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(ebitda) / SUM(total_debt_service) per L1 business segment.
+        <v xml:space="preserve">SUM(ebitda × fx_rate) / SUM(total_debt_service × fx_rate) per L1 business segment.
+Amounts converted to USD via l2.fx_rate before aggregation.
 </v>
       </c>
       <c r="AA54" t="str">

</xml_diff>

<commit_message>
Fix Number of Loans calculation at counterparty/desk/portfolio/segment levels
Three issues prevented NOL from working beyond the facility dimension:

1. Higher-level formulas queried l3.facility_exposure_calc (not loaded in
   sql.js). Rewrote all levels to COUNT DISTINCT positions directly from
   l2.position with appropriate GROUP BY.

2. adaptSql() only matched uppercase L1./L2. schema prefixes — added
   case-insensitive matching and l3 support.

3. readYamlMetricStubs() only read the first level's formula as base
   formulaSQL. Now populates formulasByDimension from all YAML levels.

Also added cross-layer fallback in loadSampleData() so L2.facility_master
resolves when sample data stores it under L1.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -6497,7 +6497,7 @@
         <v>Agg</v>
       </c>
       <c r="N66" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Counterparty_ID, lookup in Facility Table when IS(Counterparty_ID), SUM(Number_of_loans) from l3.facility_exposure_calc.
+        <v xml:space="preserve">For each Counterparty_ID, COUNT DISTINCT(Position_ID) from l2.position joined to l2.facility_master.
 </v>
       </c>
       <c r="O66" t="str">
@@ -6510,7 +6510,7 @@
         <v>Agg</v>
       </c>
       <c r="R66" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L3 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L3', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
+        <v xml:space="preserve">For each L3 LoB, COUNT DISTINCT(Position_ID) from l2.position joined to l2.facility_master and l1.enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S66" t="str">
@@ -6523,7 +6523,7 @@
         <v>Agg</v>
       </c>
       <c r="V66" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L2 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L2', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
+        <v xml:space="preserve">For each L2 LoB, COUNT DISTINCT(Position_ID) from l2.position joined to l2.facility_master and l1.enterprise_business_taxonomy hierarchy.
 </v>
       </c>
       <c r="W66" t="str">
@@ -6536,7 +6536,7 @@
         <v>Agg</v>
       </c>
       <c r="Z66" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each L1 LoB, lookup lob_segment_id from enterprise_business_taxonomy WHERE tree_level='L1', then lookup facility_id in facility_master, SUM(Number_of_loans) from l3.facility_exposure_calc.
+        <v xml:space="preserve">For each L1 LoB, COUNT DISTINCT(Position_ID) from l2.position joined to l2.facility_master and l1.enterprise_business_taxonomy hierarchy.
 </v>
       </c>
       <c r="AA66" t="str">

</xml_diff>

<commit_message>
Fix EXP-005 FX consistency bug, improve formula_text readability
- EXP-005 v2.1.0: Add missing FX rate join to counterparty/desk/portfolio/
  segment inner subqueries. Previously only facility level converted to USD;
  upper levels computed in local currency — broke cross-level reconciliation
  for multi-currency positions. Now all levels include COALESCE(fx.rate, 1).
  Verified: facility-to-segment reconciliation passes ($9.04B, diff=$0.00).
- All 5 metrics: Remove jargon ("SCD-filtered") from formula_text, replace
  with plain language ("uses current records only")
- DB-validated: 14 currencies, 1000 facilities, 452 counterparties,
  implied avg rate 2.36%, no negative values, no NULL violations

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1539,14 +1539,14 @@
         <v>EXP-005</v>
       </c>
       <c r="B14" t="str" xml:space="preserve">
-        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM.
+        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), converted to USD via FX rate and adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM via EBT hierarchy.
 </v>
       </c>
       <c r="C14" t="str">
         <v>Cost of Funds ($)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="E14" t="str">
@@ -1565,7 +1565,7 @@
         <v>Calc</v>
       </c>
       <c r="J14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="K14" t="str">
@@ -1578,7 +1578,7 @@
         <v>Agg</v>
       </c>
       <c r="N14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty: SUM of facility-level cost of funds weighted by counterparty participation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Sum each facility's cost of funds (USD, bank-share-adjusted), then weight by the counterparty's participation percentage. Aggregates across all facilities where the counterparty has a current participation record.
 </v>
       </c>
       <c r="O14" t="str">
@@ -1591,7 +1591,7 @@
         <v>Agg</v>
       </c>
       <c r="R14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L3 desk segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities assigned to each L3 desk segment in the organizational hierarchy.
 </v>
       </c>
       <c r="S14" t="str">
@@ -1604,7 +1604,7 @@
         <v>Agg</v>
       </c>
       <c r="V14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L2 portfolio segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L2 portfolio segment, traversing the EBT hierarchy from desk (L3) to portfolio (L2) via parent_segment_id.
 </v>
       </c>
       <c r="W14" t="str">
@@ -1617,7 +1617,7 @@
         <v>Agg</v>
       </c>
       <c r="Z14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L1 business segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L1 business segment, traversing the full EBT hierarchy from desk (L3) through portfolio (L2) to segment (L1).
 </v>
       </c>
       <c r="AA14" t="str">
@@ -1639,7 +1639,7 @@
         <v>Counterparty Share or Allocation (%)</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. SCD-filtered to current rows only.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="E15" t="str">
@@ -1658,7 +1658,7 @@
         <v>Raw</v>
       </c>
       <c r="J15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. SCD-filtered to current rows only.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="K15" t="str">
@@ -6837,7 +6837,7 @@
         <v>Counterparty ID</v>
       </c>
       <c r="D70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. SCD-filtered to current records only.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="E70" t="str">
@@ -6856,7 +6856,7 @@
         <v>Raw</v>
       </c>
       <c r="J70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. SCD-filtered to current records only.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="K70" t="str">
@@ -6930,7 +6930,7 @@
         <v>Counterparty Name</v>
       </c>
       <c r="D71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values returned via catalogue metadata). SCD-filtered to current records.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="E71" t="str">
@@ -6949,7 +6949,7 @@
         <v>Raw</v>
       </c>
       <c r="J71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values returned via catalogue metadata). SCD-filtered to current records.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="K71" t="str">
@@ -7023,7 +7023,7 @@
         <v>Country</v>
       </c>
       <c r="D72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). SCD-filtered to current records.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="E72" t="str">
@@ -7042,7 +7042,7 @@
         <v>Raw</v>
       </c>
       <c r="J72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). SCD-filtered to current records.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="K72" t="str">

</xml_diff>

<commit_message>
Add 5 GSIB metrics: EXP-017, EXP-018, EXP-019, EXP-020, RSK-002
- EXP-017: Undrawn Exposure ($) — unfunded commitment amount, bank-share adjusted
- EXP-018: Outstanding Exposure ($) — funded exposure via position_detail, counterparty uses attribution_pct
- EXP-019: Exposure Limit ($) — sourced from l1.limit_rule (rewritten from facility_exposure_snapshot)
- EXP-020: Exposure at Default ($) — Basel III EAD = drawn + CCF × undrawn (rewritten from L3 layer violation)
- RSK-002: Risk Rating - External Rating — numeric notch via rating_scale_dim, AVG at aggregate levels

Spec reviewed: source tables verified against DD, formulas validated
against PostgreSQL, rollup reconciliation passed (EXP-017/018/020 exact match
facility↔business_segment), GSIB risk sanity checked. 471 calc-engine tests pass.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1539,14 +1539,14 @@
         <v>EXP-005</v>
       </c>
       <c r="B14" t="str" xml:space="preserve">
-        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM.
+        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), converted to USD via FX rate and adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM via EBT hierarchy.
 </v>
       </c>
       <c r="C14" t="str">
         <v>Cost of Funds ($)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="E14" t="str">
@@ -1565,7 +1565,7 @@
         <v>Calc</v>
       </c>
       <c r="J14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="K14" t="str">
@@ -1578,7 +1578,7 @@
         <v>Agg</v>
       </c>
       <c r="N14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty: SUM of facility-level cost of funds weighted by counterparty participation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Sum each facility's cost of funds (USD, bank-share-adjusted), then weight by the counterparty's participation percentage. Aggregates across all facilities where the counterparty has a current participation record.
 </v>
       </c>
       <c r="O14" t="str">
@@ -1591,7 +1591,7 @@
         <v>Agg</v>
       </c>
       <c r="R14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L3 desk segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities assigned to each L3 desk segment in the organizational hierarchy.
 </v>
       </c>
       <c r="S14" t="str">
@@ -1604,7 +1604,7 @@
         <v>Agg</v>
       </c>
       <c r="V14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L2 portfolio segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L2 portfolio segment, traversing the EBT hierarchy from desk (L3) to portfolio (L2) via parent_segment_id.
 </v>
       </c>
       <c r="W14" t="str">
@@ -1617,7 +1617,7 @@
         <v>Agg</v>
       </c>
       <c r="Z14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L1 business segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L1 business segment, traversing the full EBT hierarchy from desk (L3) through portfolio (L2) to segment (L1).
 </v>
       </c>
       <c r="AA14" t="str">
@@ -1632,14 +1632,14 @@
         <v>EXP-006</v>
       </c>
       <c r="B15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure allocated to specific counterparty representing their share of the facility which the client can draw on. Concentration KPI measuring obligor dependency risk.
+        <v xml:space="preserve">Counterparty participation share in a facility — the percentage of a syndicated or participated facility allocated to a specific counterparty. At facility level, direct lookup from facility_counterparty_participation. At counterparty level, exposure-weighted average participation across all facilities. At desk/portfolio/segment, exposure-weighted average via EBT hierarchy. Key concentration KPI for Large Exposures Framework (LEX) and Single Counterparty Credit Limit (SCCL) compliance.
 </v>
       </c>
       <c r="C15" t="str">
         <v>Counterparty Share or Allocation (%)</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of allocation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="E15" t="str">
@@ -1658,7 +1658,7 @@
         <v>Raw</v>
       </c>
       <c r="J15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of allocation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="K15" t="str">
@@ -1668,10 +1668,10 @@
         <v>Y</v>
       </c>
       <c r="M15" t="str">
-        <v>Raw</v>
+        <v>Avg</v>
       </c>
       <c r="N15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read allocation_pct per counterparty.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities for each counterparty. Weight = drawn_amount from facility_exposure_snapshot. Falls back to simple average if no exposure data available.
 </v>
       </c>
       <c r="O15" t="str">
@@ -1681,10 +1681,10 @@
         <v>Y</v>
       </c>
       <c r="Q15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="R15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L3 desk segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S15" t="str">
@@ -1694,10 +1694,10 @@
         <v>Y</v>
       </c>
       <c r="U15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="V15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L2 portfolio segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L2 portfolio segment via enterprise_business_taxonomy hierarchy traversal.
 </v>
       </c>
       <c r="W15" t="str">
@@ -1707,10 +1707,10 @@
         <v>Y</v>
       </c>
       <c r="Y15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="Z15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L1 business segment segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L1 business segment via enterprise_business_taxonomy hierarchy traversal.
 </v>
       </c>
       <c r="AA15" t="str">
@@ -1725,14 +1725,14 @@
         <v>EXP-007</v>
       </c>
       <c r="B16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Flag identifying exposures requiring heightened monitoring due to elevated credit risk. Governance control used for enhanced monitoring, reserve consideration, and management reporting.
+        <v xml:space="preserve">Count of active Criticized risk flags across facilities. Early warning indicator of problem assets requiring heightened monitoring, reserve consideration, and management reporting. Sources from the risk_flag table filtering on flag_code = 'CRITICIZED' with uncleared status.
 </v>
       </c>
       <c r="C16" t="str">
         <v>Criticized Portfolios</v>
       </c>
       <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if criticized rating (internal_risk_rating &gt;= 6), 0 otherwise.
+        <v xml:space="preserve">For each facility, count active risk flags where flag_code = 'CRITICIZED' and the flag has not been cleared (cleared_ts IS NULL).
 </v>
       </c>
       <c r="E16" t="str">
@@ -1748,10 +1748,10 @@
         <v>Y</v>
       </c>
       <c r="I16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="J16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if criticized rating (internal_risk_rating &gt;= 6), 0 otherwise.
+        <v xml:space="preserve">For each facility, count active risk flags where flag_code = 'CRITICIZED' and the flag has not been cleared (cleared_ts IS NULL).
 </v>
       </c>
       <c r="K16" t="str">
@@ -1761,10 +1761,10 @@
         <v>Y</v>
       </c>
       <c r="M16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="N16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per counterparty.
+        <v xml:space="preserve">For each counterparty, sum facility-level criticized flag counts across all facilities belonging to that counterparty.
 </v>
       </c>
       <c r="O16" t="str">
@@ -1774,10 +1774,10 @@
         <v>Y</v>
       </c>
       <c r="Q16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="R16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L3 desk.
+        <v xml:space="preserve">Sum of criticized flag counts per L3 desk segment. Joins facility_master to enterprise_business_taxonomy via lob_segment_id.
 </v>
       </c>
       <c r="S16" t="str">
@@ -1787,10 +1787,10 @@
         <v>Y</v>
       </c>
       <c r="U16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="V16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L2 portfolio.
+        <v xml:space="preserve">Sum of criticized flag counts per L2 portfolio segment. Traverses enterprise_business_taxonomy hierarchy from L3 to L2 via parent_segment_id.
 </v>
       </c>
       <c r="W16" t="str">
@@ -1800,10 +1800,10 @@
         <v>Y</v>
       </c>
       <c r="Y16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="Z16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L1 business segment.
+        <v xml:space="preserve">Sum of criticized flag counts per L1 business segment. Full hierarchy traversal L3 → L2 → L1 via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="AA16" t="str">
@@ -1818,14 +1818,14 @@
         <v>EXP-008</v>
       </c>
       <c r="B17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Total exposure amount allocated across multiple legal entities. Supports intra-group concentration transparency.
+        <v xml:space="preserve">Total committed exposure amount (bank share) allocated across multiple legal entities for facilities flagged as cross-entity. Quantifies inter-entity concentration risk and supports intra-group transparency for GSIB reporting. Sources from counterparty_derived (L3) for the cross-entity flag and facility_exposure_snapshot (L2) for committed amounts.
 </v>
       </c>
       <c r="C17" t="str">
         <v>Cross Entity Exposure Amount</v>
       </c>
       <c r="D17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(total_cross_entity_exposure_usd) per facility from counterparty_exposure_summary. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility flagged as cross-entity, committed exposure amount weighted by the bank's participation share (bank_share_pct). Facilities without cross-entity flag are excluded.
 </v>
       </c>
       <c r="E17" t="str">
@@ -1844,7 +1844,7 @@
         <v>Agg</v>
       </c>
       <c r="J17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(total_cross_entity_exposure_usd) per facility from counterparty_exposure_summary. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility flagged as cross-entity, committed exposure amount weighted by the bank's participation share (bank_share_pct). Facilities without cross-entity flag are excluded.
 </v>
       </c>
       <c r="K17" t="str">
@@ -1857,7 +1857,7 @@
         <v>Agg</v>
       </c>
       <c r="N17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per counterparty.
+        <v xml:space="preserve">For each counterparty, sum of bank-share-weighted committed amounts across all facilities flagged as cross-entity.
 </v>
       </c>
       <c r="O17" t="str">
@@ -1870,7 +1870,7 @@
         <v>Agg</v>
       </c>
       <c r="R17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L3 desk segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S17" t="str">
@@ -1883,7 +1883,7 @@
         <v>Agg</v>
       </c>
       <c r="V17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L2 portfolio segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W17" t="str">
@@ -1896,7 +1896,7 @@
         <v>Agg</v>
       </c>
       <c r="Z17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L1 business segment segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA17" t="str">
@@ -1911,14 +1911,14 @@
         <v>EXP-009</v>
       </c>
       <c r="B18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Number of days outstanding payments is past due as grouped into 3 "buckets", 0-30 Days, 31-60 Days, 61-90+ Days. Used for staging classification and early credit deterioration monitoring.
+        <v xml:space="preserve">Maximum days payment overdue per facility, calculated from raw payment records in the payment_ledger table. For each facility, identifies payments where applied amount &lt; amount due, computes days overdue as reporting date minus payment_due_date, takes the MAX, then classifies into buckets: 1 = 0-30 days, 2 = 31-60 days, 3 = 61-90+ days. At aggregate levels, reports the worst (MAX) bucket across constituents.
 </v>
       </c>
       <c r="C18" t="str">
         <v>Days Payment Overdue Bucket</v>
       </c>
       <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID lookup the Payments records in the Payment Lockbox table, For each payment record where [Payment_Due_Date] &gt; Today() IF ([Pmt_Applied] &lt;[Pmt_Due])&gt;=1, THEN Today() - [Payment_due_date] ==[Days Overdue] SELECT MAX ([Days Overdue] then lookup in Payments Overdue bucket)
+        <v xml:space="preserve">For each facility, lookup payment records in payment_ledger where payment_due_date &lt; reporting date and payment_applied_amt &lt; payment_amount_due (underpaid). Calculate days overdue = reporting date minus payment_due_date. Take MAX days overdue, then classify into overdue bucket: 1 (0-30), 2 (31-60), 3 (61-90+).
 </v>
       </c>
       <c r="E18" t="str">
@@ -1937,7 +1937,7 @@
         <v>Calc</v>
       </c>
       <c r="J18" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID lookup the Payments records in the Payment Lockbox table, For each payment record where [Payment_Due_Date] &gt; Today() IF ([Pmt_Applied] &lt;[Pmt_Due])&gt;=1, THEN Today() - [Payment_due_date] ==[Days Overdue] SELECT MAX ([Days Overdue] then lookup in Payments Overdue bucket)
+        <v xml:space="preserve">For each facility, lookup payment records in payment_ledger where payment_due_date &lt; reporting date and payment_applied_amt &lt; payment_amount_due (underpaid). Calculate days overdue = reporting date minus payment_due_date. Take MAX days overdue, then classify into overdue bucket: 1 (0-30), 2 (31-60), 3 (61-90+).
 </v>
       </c>
       <c r="K18" t="str">
@@ -1950,7 +1950,7 @@
         <v>Agg</v>
       </c>
       <c r="N18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per counterparty.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket across all facilities per counterparty. Identifies the most severely overdue facility for each borrower.
 </v>
       </c>
       <c r="O18" t="str">
@@ -1963,7 +1963,7 @@
         <v>Agg</v>
       </c>
       <c r="R18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L3 desk segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L3 desk segment. Shows the most severe delinquency in each organizational unit.
 </v>
       </c>
       <c r="S18" t="str">
@@ -1976,7 +1976,7 @@
         <v>Agg</v>
       </c>
       <c r="V18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L2 portfolio segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W18" t="str">
@@ -1989,7 +1989,7 @@
         <v>Agg</v>
       </c>
       <c r="Z18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L1 business segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA18" t="str">
@@ -2509,14 +2509,25 @@
         <v>EXP-015</v>
       </c>
       <c r="B24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Expected Loss divided by Exposure. Derived KPI measuring loss intensity relative to exposure size, enabling comparative risk ranking across facilities or counterparties.
+        <v xml:space="preserve">Expected Loss as a percentage of committed exposure. Computed from L2 atomic risk parameters: PD (probability of default) × LGD (loss given default). At aggregate levels, uses sum-ratio rollup: SUM(PD × LGD × Committed) / SUM(Committed) × 100 — the exposure-weighted average EL rate. This ensures mathematically consistent aggregation (never averages pre-computed rates). Key credit risk quantification metric for comparing loss intensity across facilities, counterparties, and business segments.
+Ingredient derivation:
+  - PD (pd_pct): L2 facility_risk_snapshot — probability of default (%)
+  - LGD (lgd_pct): L2 facility_risk_snapshot — loss given default (%)
+  - Committed Exposure (committed_amount): L2 facility_exposure_snapshot — raw
+  - EL Rate = PD × LGD (at facility level, committed cancels in ratio)
+  - Aggregate EL Rate = SUM(PD × LGD × Committed) / SUM(Committed) × 100
 </v>
       </c>
       <c r="C24" t="str">
         <v>Expected Loss Rate (%)</v>
       </c>
       <c r="D24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of expected_loss_rate_pct per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount from l2.facility_exposure_snapshot
+  3. COMPUTE EL Rate = SUM(PD/100 × LGD/100 × Committed) / SUM(Committed) × 100
+     At facility grain, committed cancels → EL Rate ≈ PD × LGD / 100
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2)
 </v>
       </c>
       <c r="E24" t="str">
@@ -2532,10 +2543,15 @@
         <v>Y</v>
       </c>
       <c r="I24" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="J24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of expected_loss_rate_pct per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount from l2.facility_exposure_snapshot
+  3. COMPUTE EL Rate = SUM(PD/100 × LGD/100 × Committed) / SUM(Committed) × 100
+     At facility grain, committed cancels → EL Rate ≈ PD × LGD / 100
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2)
 </v>
       </c>
       <c r="K24" t="str">
@@ -2545,10 +2561,15 @@
         <v>Y</v>
       </c>
       <c r="M24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD pd_pct, lgd_pct for all facilities belonging to this counterparty
+  2. LOAD committed_amount for each facility
+  3. CONVERT to USD via l2.fx_rate spot rate
+  4. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup with FX: exposure-weighted average EL rate in USD terms.
 </v>
       </c>
       <c r="O24" t="str">
@@ -2558,10 +2579,14 @@
         <v>Y</v>
       </c>
       <c r="Q24" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="R24" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level expected_loss_rate_pct per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per desk.
 </v>
       </c>
       <c r="S24" t="str">
@@ -2571,10 +2596,14 @@
         <v>Y</v>
       </c>
       <c r="U24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per portfolio.
 </v>
       </c>
       <c r="W24" t="str">
@@ -2584,10 +2613,14 @@
         <v>Y</v>
       </c>
       <c r="Y24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per segment.
 </v>
       </c>
       <c r="AA24" t="str">
@@ -2602,14 +2635,25 @@
         <v>EXP-016</v>
       </c>
       <c r="B25" t="str" xml:space="preserve">
-        <v xml:space="preserve">PD × LGD × Exposure expressed in USD. Calculated forward-looking loss metric supporting provisioning, capital planning, and stress testing analytics.
+        <v xml:space="preserve">Expected Loss in dollar terms: PD × LGD × Committed Exposure × Bank Share. Computed from L2 atomic risk parameters and exposure data — NOT from stressed scenarios. This is the base (unstressed) expected credit loss, the foundation for provisioning, capital planning, and CECL/IFRS 9 reserve estimation.
+Ingredient derivation:
+  - PD (pd_pct): L2 facility_risk_snapshot — probability of default (%)
+  - LGD (lgd_pct): L2 facility_risk_snapshot — loss given default (%)
+  - Committed Exposure (committed_amount): L2 facility_exposure_snapshot — raw
+  - Bank Share (bank_share_pct): L2 facility_exposure_snapshot — participation %
+  - EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Rollup uses direct-sum: SUM(facility EL) at each aggregate level. FX conversion applied at aggregate levels for multi-currency portfolios.
 </v>
       </c>
       <c r="C25" t="str">
         <v>Expected Loss ($)</v>
       </c>
       <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount, bank_share_pct from l2.facility_exposure_snapshot
+  3. COMPUTE EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2), bank_share_pct (L2)
 </v>
       </c>
       <c r="E25" t="str">
@@ -2625,10 +2669,14 @@
         <v>Y</v>
       </c>
       <c r="I25" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="J25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount, bank_share_pct from l2.facility_exposure_snapshot
+  3. COMPUTE EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2), bank_share_pct (L2)
 </v>
       </c>
       <c r="K25" t="str">
@@ -2641,7 +2689,11 @@
         <v>Agg</v>
       </c>
       <c r="N25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD facility-level EL for all facilities of this counterparty
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) = Counterparty EL (USD)
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="O25" t="str">
@@ -2654,7 +2706,11 @@
         <v>Agg</v>
       </c>
       <c r="R25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per desk
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="S25" t="str">
@@ -2667,7 +2723,11 @@
         <v>Agg</v>
       </c>
       <c r="V25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per portfolio
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="W25" t="str">
@@ -2680,7 +2740,11 @@
         <v>Agg</v>
       </c>
       <c r="Z25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per business segment
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="AA25" t="str">
@@ -2702,11 +2766,21 @@
         <v>Undrawn Exposure ($)</v>
       </c>
       <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
-2. Subtract from committed_facility_amt to get unfunded amount
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
-Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY fm.facility_id
+6. COMPUTE
+   metric_value = (committed_facility_amt - SUM(funded_amount))
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="E26" t="str">
@@ -2725,11 +2799,21 @@
         <v>Calc</v>
       </c>
       <c r="J26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
-2. Subtract from committed_facility_amt to get unfunded amount
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
-Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY fm.facility_id
+6. COMPUTE
+   metric_value = (committed_facility_amt - SUM(funded_amount))
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="K26" t="str">
@@ -2742,8 +2826,13 @@
         <v>Calc</v>
       </c>
       <c r="N26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty, sum facility-level undrawn exposure weighted
-by participation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_counterparty_participation  (fcp)
+   ON    fcp.facility_id = fac.facility_id
+   AND   fcp.is_current_flag = 'Y'
+3. GROUP BY fcp.counterparty_id
+4. COMPUTE
+   metric_value = SUM(facility_undrawn * participation_pct)
 </v>
       </c>
       <c r="O26" t="str">
@@ -2756,8 +2845,15 @@
         <v>Agg</v>
       </c>
       <c r="R26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L3 desk segment.
-Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="S26" t="str">
@@ -2770,8 +2866,16 @@
         <v>Agg</v>
       </c>
       <c r="V26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L2 portfolio segment.
-Traverses L3 -&gt; L2 via parent_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="W26" t="str">
@@ -2784,8 +2888,18 @@
         <v>Agg</v>
       </c>
       <c r="Z26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L1 business segment.
-Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l1)
+   ON    ebt_l1.managed_segment_id = ebt_l2.parent_segment_id
+6. GROUP BY ebt_l1.managed_segment_id
+7. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="AA26" t="str">
@@ -2800,17 +2914,28 @@
         <v>EXP-018</v>
       </c>
       <c r="B27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Bank-share-adjusted funded (drawn) exposure amount. Represents the portion of committed credit currently utilized by the borrower. Maps to FR Y-14Q Field 25 (Utilized Exposure Global, MDRM G075).
+        <v xml:space="preserve">Bank-share-adjusted funded (drawn) exposure amount. Represents the portion of committed credit currently utilized by the borrower. Maps to FR Y-14Q Field 25 (Utilized Exposure Global, MDRM G075). Counterparty level uses exposure_counterparty_attribution for risk-shifted attribution weighting per Basel III requirements.
 </v>
       </c>
       <c r="C27" t="str">
         <v>Outstanding Exposure ($)</v>
       </c>
       <c r="D27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(funded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY pos.facility_id
+6. COMPUTE
+   metric_value = SUM(funded_amount)
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="E27" t="str">
@@ -2829,10 +2954,21 @@
         <v>Calc</v>
       </c>
       <c r="J27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(funded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY pos.facility_id
+6. COMPUTE
+   metric_value = SUM(funded_amount)
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="K27" t="str">
@@ -2845,9 +2981,13 @@
         <v>Calc</v>
       </c>
       <c r="N27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty, sum facility-level outstanding exposure weighted
-by participation_pct from facility_counterparty_participation.
-Uses contractual pro-rata basis per FR Y-14Q requirements.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.exposure_counterparty_attribution  (eca)
+   ON    eca.facility_id = fac.facility_id
+   AND   eca.as_of_date = :as_of_date
+3. GROUP BY eca.counterparty_id
+4. COMPUTE
+   metric_value = SUM(facility_outstanding * attribution_pct)
 </v>
       </c>
       <c r="O27" t="str">
@@ -2860,8 +3000,15 @@
         <v>Agg</v>
       </c>
       <c r="R27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L3 desk segment.
-Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="S27" t="str">
@@ -2874,8 +3021,16 @@
         <v>Agg</v>
       </c>
       <c r="V27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L2 portfolio segment.
-Traverses L3 -&gt; L2 via parent_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="W27" t="str">
@@ -2888,8 +3043,14 @@
         <v>Agg</v>
       </c>
       <c r="Z27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L1 business segment.
-Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+4. GROUP BY ebt_l1.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="AA27" t="str">
@@ -2904,14 +3065,15 @@
         <v>EXP-019</v>
       </c>
       <c r="B28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Maximum approved credit exposure authorized for the counterparty or Line of Business segment in USD. Represents formal risk appetite allocation and governance control threshold.
+        <v xml:space="preserve">Maximum approved credit exposure authorized for the counterparty or Line of Business segment in USD. Sourced directly from the limit_rule reference table. Represents formal risk appetite allocation and governance control threshold set by the Credit Risk Committee. Not applicable at individual facility level — limits are set at counterparty and organizational hierarchy levels.
 </v>
       </c>
       <c r="C28" t="str">
         <v>Exposure Limit ($)</v>
       </c>
       <c r="D28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt from lob_exposure_summary for each facility as-of reporting date.
+        <v xml:space="preserve">Not applicable — exposure limits are set at counterparty and
+organizational levels, not per individual facility. Returns NULL.
 </v>
       </c>
       <c r="E28" t="str">
@@ -2930,7 +3092,8 @@
         <v>Raw</v>
       </c>
       <c r="J28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt from lob_exposure_summary for each facility as-of reporting date.
+        <v xml:space="preserve">Not applicable — exposure limits are set at counterparty and
+organizational levels, not per individual facility. Returns NULL.
 </v>
       </c>
       <c r="K28" t="str">
@@ -2943,7 +3106,12 @@
         <v>Raw</v>
       </c>
       <c r="N28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt per counterparty.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.counterparty_id IS NOT NULL
+2. GROUP BY lr.counterparty_id
+3. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="O28" t="str">
@@ -2953,10 +3121,18 @@
         <v>Y</v>
       </c>
       <c r="Q28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="R28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="S28" t="str">
@@ -2966,10 +3142,18 @@
         <v>Y</v>
       </c>
       <c r="U28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="V28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="W28" t="str">
@@ -2979,10 +3163,18 @@
         <v>Y</v>
       </c>
       <c r="Y28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="Z28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="AA28" t="str">
@@ -2997,14 +3189,25 @@
         <v>EXP-020</v>
       </c>
       <c r="B29" t="str" xml:space="preserve">
-        <v xml:space="preserve">The estimated exposure amount (in USD) expected to be outstanding if the borrower defaults.
+        <v xml:space="preserve">Estimated exposure amount outstanding if the borrower defaults, computed from L2 atomic inputs per Basel III: EAD = OB + CCF × Undrawn, where OB = drawn/funded amount, CCF = credit conversion factor from facility_risk_snapshot, and Undrawn = committed minus drawn from facility_exposure_snapshot. Bank-share adjusted via facility_exposure_snapshot. At counterparty level, weighted by participation_pct from facility_counterparty_participation per FR Y-14Q requirements.
 </v>
       </c>
       <c r="C29" t="str">
         <v>Exposure at Default ($)</v>
       </c>
       <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read exposure_at_default from credit_event_facility_link for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+   AND   frs.as_of_date = fes.as_of_date
+4. GROUP BY fes.facility_id
+5. COMPUTE
+   metric_value = (drawn_amount + CCF * undrawn_amount)
+                  * bank_share_pct / 100
 </v>
       </c>
       <c r="E29" t="str">
@@ -3020,10 +3223,21 @@
         <v>Y</v>
       </c>
       <c r="I29" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="J29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read exposure_at_default from credit_event_facility_link for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+   AND   frs.as_of_date = fes.as_of_date
+4. GROUP BY fes.facility_id
+5. COMPUTE
+   metric_value = (drawn_amount + CCF * undrawn_amount)
+                  * bank_share_pct / 100
 </v>
       </c>
       <c r="K29" t="str">
@@ -3033,10 +3247,22 @@
         <v>Y</v>
       </c>
       <c r="M29" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per counterparty.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+4. JOIN  l2.facility_counterparty_participation  (fcp)
+   ON    fcp.facility_id = fes.facility_id
+   AND   fcp.is_current_flag = 'Y'
+5. GROUP BY fcp.counterparty_id
+6. COMPUTE
+   metric_value = SUM((drawn + CCF * undrawn) * bank_share / 100
+                  * participation_pct)
 </v>
       </c>
       <c r="O29" t="str">
@@ -3049,7 +3275,15 @@
         <v>Agg</v>
       </c>
       <c r="R29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="S29" t="str">
@@ -3062,7 +3296,13 @@
         <v>Agg</v>
       </c>
       <c r="V29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2)
+   Traverse L3 -&gt; L2 via parent_segment_id
+4. GROUP BY ebt_l2.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="W29" t="str">
@@ -3075,7 +3315,13 @@
         <v>Agg</v>
       </c>
       <c r="Z29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+4. GROUP BY ebt_l1.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="AA29" t="str">
@@ -5796,14 +6042,15 @@
         <v>PRC-003</v>
       </c>
       <c r="B59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of exposures within portfolio with approved pricing or policy exceptions. Derived governance KPI measuring policy discipline and risk culture strength.
+        <v xml:space="preserve">Percentage of facilities with approved pricing or policy exceptions. Computed as COUNT(exception facilities) / COUNT(total facilities) × 100. Sourced from L2 facility_pricing_snapshot — the atomic pricing record — using the is_pricing_exception_flag. At aggregate levels, uses count-ratio rollup: re-counts exceptions and totals across all constituent facilities, never averages pre-computed rates. Key governance KPI measuring policy discipline, risk culture strength, and pricing override frequency.
 </v>
       </c>
       <c r="C59" t="str">
         <v>Exception Rate (%)</v>
       </c>
       <c r="D59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if pricing exception, 0 otherwise.
+        <v xml:space="preserve">Binary flag: 1.0 if pricing exception approved, 0.0 otherwise.
+Ingredients: is_pricing_exception_flag (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="E59" t="str">
@@ -5822,7 +6069,8 @@
         <v>Calc</v>
       </c>
       <c r="J59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if pricing exception, 0 otherwise.
+        <v xml:space="preserve">Binary flag: 1.0 if pricing exception approved, 0.0 otherwise.
+Ingredients: is_pricing_exception_flag (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="K59" t="str">
@@ -5835,7 +6083,10 @@
         <v>Calc</v>
       </c>
       <c r="N59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD is_pricing_exception_flag for all facilities of this counterparty
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup: re-counts from facility-level flags.
 </v>
       </c>
       <c r="O59" t="str">
@@ -5848,7 +6099,10 @@
         <v>Calc</v>
       </c>
       <c r="R59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L3 desk.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per desk.
 </v>
       </c>
       <c r="S59" t="str">
@@ -5861,7 +6115,10 @@
         <v>Calc</v>
       </c>
       <c r="V59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L2 portfolio.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per portfolio.
 </v>
       </c>
       <c r="W59" t="str">
@@ -5874,7 +6131,10 @@
         <v>Calc</v>
       </c>
       <c r="Z59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L1 business segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per business segment.
 </v>
       </c>
       <c r="AA59" t="str">
@@ -6830,14 +7090,14 @@
         <v>REF-004</v>
       </c>
       <c r="B70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Unique system identifier assigned to the borrower or obligor. Used for exposure aggregation and risk consolidation.
+        <v xml:space="preserve">Unique system identifier assigned to the borrower or obligor. Used for exposure aggregation and risk consolidation across the GSIB. At facility level, returns the counterparty_id linked to each facility. At upper levels, returns COUNT(DISTINCT counterparty_id) — the number of unique obligors in each organizational segment.
 </v>
       </c>
       <c r="C70" t="str">
         <v>Counterparty ID</v>
       </c>
       <c r="D70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="E70" t="str">
@@ -6856,7 +7116,7 @@
         <v>Raw</v>
       </c>
       <c r="J70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="K70" t="str">
@@ -6869,7 +7129,7 @@
         <v>Raw</v>
       </c>
       <c r="N70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Identity — returns counterparty_id for each current counterparty.
 </v>
       </c>
       <c r="O70" t="str">
@@ -6882,7 +7142,7 @@
         <v>Agg</v>
       </c>
       <c r="R70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L3 desk segment — number of unique obligors in each desk.
 </v>
       </c>
       <c r="S70" t="str">
@@ -6895,7 +7155,7 @@
         <v>Agg</v>
       </c>
       <c r="V70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L2 portfolio segment — number of unique obligors in each portfolio.
 </v>
       </c>
       <c r="W70" t="str">
@@ -6908,7 +7168,7 @@
         <v>Agg</v>
       </c>
       <c r="Z70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L1 business segment segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L1 business segment — number of unique obligors in each business segment.
 </v>
       </c>
       <c r="AA70" t="str">
@@ -6923,14 +7183,14 @@
         <v>REF-005</v>
       </c>
       <c r="B71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Descriptive name of the counterparty as documented in the credit agreement. Used for reporting clarity and operational reference.
+        <v xml:space="preserve">Legal name of the counterparty as documented in the credit agreement. At facility level, returns the counterparty_id (numeric proxy for the name since metric values are numeric). At counterparty level, identity lookup. At upper levels, COUNT(DISTINCT counterparty_id) — number of unique named obligors per organizational segment. Used for reporting clarity and operational reference across all regulatory submissions.
 </v>
       </c>
       <c r="C71" t="str">
         <v>Counterparty Name</v>
       </c>
       <c r="D71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_name from counterparty for each facility's counterparty.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="E71" t="str">
@@ -6949,7 +7209,7 @@
         <v>Raw</v>
       </c>
       <c r="J71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_name from counterparty for each facility's counterparty.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="K71" t="str">
@@ -6959,10 +7219,10 @@
         <v>Y</v>
       </c>
       <c r="M71" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="N71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per counterparty.
+        <v xml:space="preserve">Identity — returns counterparty_id for each current counterparty. Legal name resolved via counterparty dimension join at display time.
 </v>
       </c>
       <c r="O71" t="str">
@@ -6975,7 +7235,7 @@
         <v>Agg</v>
       </c>
       <c r="R71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L3 desk segment — number of unique named obligors in each desk.
 </v>
       </c>
       <c r="S71" t="str">
@@ -6988,7 +7248,7 @@
         <v>Agg</v>
       </c>
       <c r="V71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L2 portfolio segment — number of unique named obligors in each portfolio.
 </v>
       </c>
       <c r="W71" t="str">
@@ -7001,7 +7261,7 @@
         <v>Agg</v>
       </c>
       <c r="Z71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L1 business segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L1 business segment — number of unique named obligors in each business segment.
 </v>
       </c>
       <c r="AA71" t="str">
@@ -7016,14 +7276,14 @@
         <v>REF-006</v>
       </c>
       <c r="B72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Country of risk or booking location. Supports geographic concentration and sovereign risk analysis.
+        <v xml:space="preserve">Country of risk derived from the counterparty's domicile. At facility level, returns a numeric country identifier (via counterparty → country_dim join path). At counterparty level, identity lookup. At desk/portfolio/segment levels, COUNT(DISTINCT country_code) — geographic diversification indicator showing the number of unique countries represented. Supports FFIEC 009 Country Exposure Report and Basel III geographic concentration analysis.
 </v>
       </c>
       <c r="C72" t="str">
         <v>Country</v>
       </c>
       <c r="D72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of country_name from country_dim.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="E72" t="str">
@@ -7042,7 +7302,7 @@
         <v>Raw</v>
       </c>
       <c r="J72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of country_name from country_dim.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="K72" t="str">
@@ -7055,7 +7315,7 @@
         <v>Raw</v>
       </c>
       <c r="N72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read country_name per counterparty.
+        <v xml:space="preserve">Lookup country for each counterparty via country_code → country_dim join. Returns counterparty_id as numeric proxy.
 </v>
       </c>
       <c r="O72" t="str">
@@ -7068,7 +7328,7 @@
         <v>Agg</v>
       </c>
       <c r="R72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L3 desk segment — number of unique countries represented, a geographic diversification indicator.
 </v>
       </c>
       <c r="S72" t="str">
@@ -7081,7 +7341,7 @@
         <v>Agg</v>
       </c>
       <c r="V72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L2 portfolio segment — number of unique countries represented in each portfolio.
 </v>
       </c>
       <c r="W72" t="str">
@@ -7094,7 +7354,7 @@
         <v>Agg</v>
       </c>
       <c r="Z72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L1 business segment segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L1 business segment — geographic diversification at the highest organizational level.
 </v>
       </c>
       <c r="AA72" t="str">
@@ -7109,14 +7369,14 @@
         <v>REF-007</v>
       </c>
       <c r="B73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Unique identifier linking facility to governing credit agreement documentation.
+        <v xml:space="preserve">Unique identifier linking each facility to its governing credit agreement documentation. Used for contract tracking, facility-to-agreement linkage, and regulatory reporting. At counterparty level, returns count of distinct credit agreements per borrower.
 </v>
       </c>
       <c r="C73" t="str">
         <v>Credit Agreement ID</v>
       </c>
       <c r="D73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of credit_agreement_id from credit_agreement_master.
+        <v xml:space="preserve">Direct lookup of credit_agreement_id for each active facility via facility_master joined to credit_agreement_master.
 </v>
       </c>
       <c r="E73" t="str">
@@ -7135,7 +7395,7 @@
         <v>Raw</v>
       </c>
       <c r="J73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of credit_agreement_id from credit_agreement_master.
+        <v xml:space="preserve">Direct lookup of credit_agreement_id for each active facility via facility_master joined to credit_agreement_master.
 </v>
       </c>
       <c r="K73" t="str">
@@ -7145,10 +7405,10 @@
         <v>Y</v>
       </c>
       <c r="M73" t="str">
-        <v>Raw</v>
+        <v>Agg</v>
       </c>
       <c r="N73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read credit_agreement_id per counterparty.
+        <v xml:space="preserve">Count of distinct credit agreements per counterparty. Provides visibility into borrower complexity and multi-agreement relationships.
 </v>
       </c>
       <c r="O73" t="str">
@@ -7161,7 +7421,7 @@
         <v>Agg</v>
       </c>
       <c r="R73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L3 desk segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S73" t="str">
@@ -7174,7 +7434,7 @@
         <v>Agg</v>
       </c>
       <c r="V73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L2 portfolio segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W73" t="str">
@@ -7187,7 +7447,7 @@
         <v>Agg</v>
       </c>
       <c r="Z73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L1 business segment segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA73" t="str">
@@ -7295,7 +7555,7 @@
         <v>REF-009</v>
       </c>
       <c r="B75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Date on which loan or contract became legally effective.
+        <v xml:space="preserve">Date on which loan or contract became legally effective. Sourced directly from facility_master. At aggregate levels, returns the earliest origination date (MIN) across constituent facilities — indicating the oldest vintage in the book. Key contract lifecycle tracking attribute for vintage analysis and portfolio seasoning assessment.
 </v>
       </c>
       <c r="C75" t="str">
@@ -7303,6 +7563,7 @@
       </c>
       <c r="D75" t="str" xml:space="preserve">
         <v xml:space="preserve">Direct lookup of origination_date from facility_master.
+Ingredients: origination_date (L2 facility_master — raw field)
 </v>
       </c>
       <c r="E75" t="str">
@@ -7322,6 +7583,7 @@
       </c>
       <c r="J75" t="str" xml:space="preserve">
         <v xml:space="preserve">Direct lookup of origination_date from facility_master.
+Ingredients: origination_date (L2 facility_master — raw field)
 </v>
       </c>
       <c r="K75" t="str">
@@ -7334,7 +7596,10 @@
         <v>Agg</v>
       </c>
       <c r="N75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level origination_date) per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD origination_date from l2.facility_master for all active facilities
+  2. COMPUTE MIN(origination_date) — earliest contract vintage
+Indicates the oldest banking relationship tenure for this counterparty.
 </v>
       </c>
       <c r="O75" t="str">
@@ -7347,7 +7612,10 @@
         <v>Agg</v>
       </c>
       <c r="R75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOAD origination_date from l2.facility_master
+  2. JOIN l1.enterprise_business_taxonomy on lob_segment_id
+  3. COMPUTE MIN(origination_date) — earliest vintage in desk book
 </v>
       </c>
       <c r="S75" t="str">
@@ -7360,7 +7628,9 @@
         <v>Agg</v>
       </c>
       <c r="V75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE MIN(origination_date) — earliest vintage in portfolio
 </v>
       </c>
       <c r="W75" t="str">
@@ -7373,7 +7643,9 @@
         <v>Agg</v>
       </c>
       <c r="Z75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE MIN(origination_date) — earliest vintage in business segment
 </v>
       </c>
       <c r="AA75" t="str">
@@ -9620,14 +9892,14 @@
         <v>RSK-001</v>
       </c>
       <c r="B100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Most recent internal credit rating assigned at reporting date. Used for segmentation and exposure-weighted risk aggregation.
+        <v xml:space="preserve">Risk rating tier derived from counterparty probability of default (PD). Each counterparty's pd_annual is matched against the risk_rating_tier_dim reference table (pd_min_pct / pd_max_pct boundaries) to assign a tier classification. At facility level, the tier is inherited from the owning counterparty. At aggregate levels, MAX (worst-case) tier ordinal is reported.
 </v>
       </c>
       <c r="C100" t="str">
         <v>Risk Rating Tier</v>
       </c>
       <c r="D100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read risk_rating_status from counterparty_rating_observation for each facility.
+        <v xml:space="preserve">For each facility, inherit the risk rating tier from the owning counterparty. Join facility_master to counterparty, then range-match counterparty pd_annual against risk_rating_tier_dim to derive the tier ordinal (display_order).
 </v>
       </c>
       <c r="E100" t="str">
@@ -9643,10 +9915,10 @@
         <v>Y</v>
       </c>
       <c r="I100" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="J100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read risk_rating_status from counterparty_rating_observation for each facility.
+        <v xml:space="preserve">For each facility, inherit the risk rating tier from the owning counterparty. Join facility_master to counterparty, then range-match counterparty pd_annual against risk_rating_tier_dim to derive the tier ordinal (display_order).
 </v>
       </c>
       <c r="K100" t="str">
@@ -9656,10 +9928,10 @@
         <v>Y</v>
       </c>
       <c r="M100" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per counterparty.
+        <v xml:space="preserve">For each counterparty, look up pd_annual and range-match against risk_rating_tier_dim where pd_annual &gt;= pd_min_pct AND pd_annual &lt; pd_max_pct. Returns the tier ordinal (display_order). Counterparties with NULL PD receive tier 0 (unrated).
 </v>
       </c>
       <c r="O100" t="str">
@@ -9672,7 +9944,7 @@
         <v>Agg</v>
       </c>
       <c r="R100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L3 desk segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal across all counterparties in the L3 desk segment. Higher ordinal = riskier tier. Full tier distribution available via counterparty-level drill-down.
 </v>
       </c>
       <c r="S100" t="str">
@@ -9685,7 +9957,7 @@
         <v>Agg</v>
       </c>
       <c r="V100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L2 portfolio segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W100" t="str">
@@ -9698,7 +9970,7 @@
         <v>Agg</v>
       </c>
       <c r="Z100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L1 business segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA100" t="str">
@@ -9713,14 +9985,23 @@
         <v>RSK-002</v>
       </c>
       <c r="B101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Current external credit agency rating assigned to the obligor. Used for benchmarking, regulatory reporting, and external credit risk validation. Sourced based on external Rating provider (S&amp;P, Moodys, Fitch) - populated based on firm's preferred recognized rating provider.
+        <v xml:space="preserve">External credit agency rating expressed as a numeric notch value from the rating_scale_dim. At facility/counterparty levels, returns the raw notch of the external rating. At aggregate levels (desk, portfolio, segment), computes the exposure-weighted average notch across all positions, rounded to the nearest whole notch. Lower notch = better rating (e.g., 1=AAA, 21=D). Sourced from position.external_risk_rating, mapped to rating_scale_dim.rating_value.
 </v>
       </c>
       <c r="C101" t="str">
         <v>Risk Rating - External Rating</v>
       </c>
       <c r="D101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating from position for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+   AND   rs.is_current_flag = 'Y'
+4. COMPUTE
+   metric_value = rs.rating_value
 </v>
       </c>
       <c r="E101" t="str">
@@ -9739,7 +10020,16 @@
         <v>Raw</v>
       </c>
       <c r="J101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating from position for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+   AND   rs.is_current_flag = 'Y'
+4. COMPUTE
+   metric_value = rs.rating_value
 </v>
       </c>
       <c r="K101" t="str">
@@ -9752,7 +10042,15 @@
         <v>Raw</v>
       </c>
       <c r="N101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating per counterparty.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. GROUP BY fm.counterparty_id
+5. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="O101" t="str">
@@ -9762,10 +10060,20 @@
         <v>Y</v>
       </c>
       <c r="Q101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="R101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+5. GROUP BY ebt.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="S101" t="str">
@@ -9775,10 +10083,19 @@
         <v>Y</v>
       </c>
       <c r="U101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="V101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2)
+   Traverse L3 -&gt; L2 via parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="W101" t="str">
@@ -9788,10 +10105,19 @@
         <v>Y</v>
       </c>
       <c r="Y101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="Z101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+5. GROUP BY ebt_l1.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="AA101" t="str">

</xml_diff>

<commit_message>
Activate 5 GSIB metrics: REF-009, REF-024, PRC-009, PRC-006, EXP-030
- REF-009: Facility Origination Date — enhanced with portfolio-level
  pipeline count (inactive facilities approaching activation)
- REF-024: Participating Counterparty IDs — fixed from SUM(IDs) to
  COUNT(DISTINCT counterparty_id) at aggregate levels
- PRC-009: Pricing Exception Status — fixed L3→L2 sourcing, added
  ordinal status encoding + count-ratio aggregate rollup
- PRC-006: Pricing Tier — fixed L3→L2 sourcing, range-join spread_bps
  against pricing_tier_dim, exposure-weighted avg at aggregate levels
- EXP-030: Probability of Default (%) — fixed weighted-avg formula
  SUM(PD×committed)/SUM(committed) consistently at all levels

Spec reviewed: source tables verified against DD, formulas validated
against PostgreSQL, rollup reconciliation passed, GSIB risk sanity checked.
All 458 calc-engine tests pass.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -1539,14 +1539,14 @@
         <v>EXP-005</v>
       </c>
       <c r="B14" t="str" xml:space="preserve">
-        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM.
+        <v xml:space="preserve">The portion of total funding-related expense attributed to a specific exposure or portfolio. At facility level, calculated as SUM across all positions of (funded_amount * interest_rate), converted to USD via FX rate and adjusted for bank share. At counterparty level, further adjusted by counterparty participation_pct. At desk/portfolio/segment levels, aggregated as SUM via EBT hierarchy.
 </v>
       </c>
       <c r="C14" t="str">
         <v>Cost of Funds ($)</v>
       </c>
       <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="E14" t="str">
@@ -1565,7 +1565,7 @@
         <v>Calc</v>
       </c>
       <c r="J14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each position under the facility: funded_amount * interest_rate = Position Cost of Funds. Adjusted by bank_share: SUM(funded_amount * interest_rate) * bank_share_pct / 100. Joins position_detail → position (for facility_id) → facility_master.
+        <v xml:space="preserve">For each position under the facility, compute funded_amount x interest_rate, convert to USD using the FX spot rate (defaults to 1.0 for USD positions). Sum across all positions, then multiply by the bank's share percentage. Result = annual cost of funds for this facility in USD.
 </v>
       </c>
       <c r="K14" t="str">
@@ -1578,7 +1578,7 @@
         <v>Agg</v>
       </c>
       <c r="N14" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty: SUM of facility-level cost of funds weighted by counterparty participation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Sum each facility's cost of funds (USD, bank-share-adjusted), then weight by the counterparty's participation percentage. Aggregates across all facilities where the counterparty has a current participation record.
 </v>
       </c>
       <c r="O14" t="str">
@@ -1591,7 +1591,7 @@
         <v>Agg</v>
       </c>
       <c r="R14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L3 desk segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities assigned to each L3 desk segment in the organizational hierarchy.
 </v>
       </c>
       <c r="S14" t="str">
@@ -1604,7 +1604,7 @@
         <v>Agg</v>
       </c>
       <c r="V14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L2 portfolio segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L2 portfolio segment, traversing the EBT hierarchy from desk (L3) to portfolio (L2) via parent_segment_id.
 </v>
       </c>
       <c r="W14" t="str">
@@ -1617,7 +1617,7 @@
         <v>Agg</v>
       </c>
       <c r="Z14" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level cost of funds (bank-share-adjusted) per L1 business segment.
+        <v xml:space="preserve">Sum of facility-level cost of funds (USD, bank-share-adjusted) for all facilities within each L1 business segment, traversing the full EBT hierarchy from desk (L3) through portfolio (L2) to segment (L1).
 </v>
       </c>
       <c r="AA14" t="str">
@@ -1632,14 +1632,14 @@
         <v>EXP-006</v>
       </c>
       <c r="B15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure allocated to specific counterparty representing their share of the facility which the client can draw on. Concentration KPI measuring obligor dependency risk.
+        <v xml:space="preserve">Counterparty participation share in a facility — the percentage of a syndicated or participated facility allocated to a specific counterparty. At facility level, direct lookup from facility_counterparty_participation. At counterparty level, exposure-weighted average participation across all facilities. At desk/portfolio/segment, exposure-weighted average via EBT hierarchy. Key concentration KPI for Large Exposures Framework (LEX) and Single Counterparty Credit Limit (SCCL) compliance.
 </v>
       </c>
       <c r="C15" t="str">
         <v>Counterparty Share or Allocation (%)</v>
       </c>
       <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of allocation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="E15" t="str">
@@ -1658,7 +1658,7 @@
         <v>Raw</v>
       </c>
       <c r="J15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of allocation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">Direct lookup of participation_pct from facility_counterparty_participation for the primary counterparty on each facility. Uses current records only.
 </v>
       </c>
       <c r="K15" t="str">
@@ -1668,10 +1668,10 @@
         <v>Y</v>
       </c>
       <c r="M15" t="str">
-        <v>Raw</v>
+        <v>Avg</v>
       </c>
       <c r="N15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read allocation_pct per counterparty.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities for each counterparty. Weight = drawn_amount from facility_exposure_snapshot. Falls back to simple average if no exposure data available.
 </v>
       </c>
       <c r="O15" t="str">
@@ -1681,10 +1681,10 @@
         <v>Y</v>
       </c>
       <c r="Q15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="R15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L3 desk segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S15" t="str">
@@ -1694,10 +1694,10 @@
         <v>Y</v>
       </c>
       <c r="U15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="V15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L2 portfolio segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L2 portfolio segment via enterprise_business_taxonomy hierarchy traversal.
 </v>
       </c>
       <c r="W15" t="str">
@@ -1707,10 +1707,10 @@
         <v>Y</v>
       </c>
       <c r="Y15" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="Z15" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level allocation_pct per L1 business segment segment.
+        <v xml:space="preserve">Exposure-weighted average participation across all facilities per L1 business segment via enterprise_business_taxonomy hierarchy traversal.
 </v>
       </c>
       <c r="AA15" t="str">
@@ -1725,14 +1725,14 @@
         <v>EXP-007</v>
       </c>
       <c r="B16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Flag identifying exposures requiring heightened monitoring due to elevated credit risk. Governance control used for enhanced monitoring, reserve consideration, and management reporting.
+        <v xml:space="preserve">Count of active Criticized risk flags across facilities. Early warning indicator of problem assets requiring heightened monitoring, reserve consideration, and management reporting. Sources from the risk_flag table filtering on flag_code = 'CRITICIZED' with uncleared status.
 </v>
       </c>
       <c r="C16" t="str">
         <v>Criticized Portfolios</v>
       </c>
       <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if criticized rating (internal_risk_rating &gt;= 6), 0 otherwise.
+        <v xml:space="preserve">For each facility, count active risk flags where flag_code = 'CRITICIZED' and the flag has not been cleared (cleared_ts IS NULL).
 </v>
       </c>
       <c r="E16" t="str">
@@ -1748,10 +1748,10 @@
         <v>Y</v>
       </c>
       <c r="I16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="J16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if criticized rating (internal_risk_rating &gt;= 6), 0 otherwise.
+        <v xml:space="preserve">For each facility, count active risk flags where flag_code = 'CRITICIZED' and the flag has not been cleared (cleared_ts IS NULL).
 </v>
       </c>
       <c r="K16" t="str">
@@ -1761,10 +1761,10 @@
         <v>Y</v>
       </c>
       <c r="M16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="N16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per counterparty.
+        <v xml:space="preserve">For each counterparty, sum facility-level criticized flag counts across all facilities belonging to that counterparty.
 </v>
       </c>
       <c r="O16" t="str">
@@ -1774,10 +1774,10 @@
         <v>Y</v>
       </c>
       <c r="Q16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="R16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L3 desk.
+        <v xml:space="preserve">Sum of criticized flag counts per L3 desk segment. Joins facility_master to enterprise_business_taxonomy via lob_segment_id.
 </v>
       </c>
       <c r="S16" t="str">
@@ -1787,10 +1787,10 @@
         <v>Y</v>
       </c>
       <c r="U16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="V16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L2 portfolio.
+        <v xml:space="preserve">Sum of criticized flag counts per L2 portfolio segment. Traverses enterprise_business_taxonomy hierarchy from L3 to L2 via parent_segment_id.
 </v>
       </c>
       <c r="W16" t="str">
@@ -1800,10 +1800,10 @@
         <v>Y</v>
       </c>
       <c r="Y16" t="str">
-        <v>Calc</v>
+        <v>Agg</v>
       </c>
       <c r="Z16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with criticized rating (internal_risk_rating &gt;= 6) per L1 business segment.
+        <v xml:space="preserve">Sum of criticized flag counts per L1 business segment. Full hierarchy traversal L3 → L2 → L1 via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="AA16" t="str">
@@ -1818,14 +1818,14 @@
         <v>EXP-008</v>
       </c>
       <c r="B17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Total exposure amount allocated across multiple legal entities. Supports intra-group concentration transparency.
+        <v xml:space="preserve">Total committed exposure amount (bank share) allocated across multiple legal entities for facilities flagged as cross-entity. Quantifies inter-entity concentration risk and supports intra-group transparency for GSIB reporting. Sources from counterparty_derived (L3) for the cross-entity flag and facility_exposure_snapshot (L2) for committed amounts.
 </v>
       </c>
       <c r="C17" t="str">
         <v>Cross Entity Exposure Amount</v>
       </c>
       <c r="D17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(total_cross_entity_exposure_usd) per facility from counterparty_exposure_summary. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility flagged as cross-entity, committed exposure amount weighted by the bank's participation share (bank_share_pct). Facilities without cross-entity flag are excluded.
 </v>
       </c>
       <c r="E17" t="str">
@@ -1844,7 +1844,7 @@
         <v>Agg</v>
       </c>
       <c r="J17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(total_cross_entity_exposure_usd) per facility from counterparty_exposure_summary. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility flagged as cross-entity, committed exposure amount weighted by the bank's participation share (bank_share_pct). Facilities without cross-entity flag are excluded.
 </v>
       </c>
       <c r="K17" t="str">
@@ -1857,7 +1857,7 @@
         <v>Agg</v>
       </c>
       <c r="N17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per counterparty.
+        <v xml:space="preserve">For each counterparty, sum of bank-share-weighted committed amounts across all facilities flagged as cross-entity.
 </v>
       </c>
       <c r="O17" t="str">
@@ -1870,7 +1870,7 @@
         <v>Agg</v>
       </c>
       <c r="R17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L3 desk segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S17" t="str">
@@ -1883,7 +1883,7 @@
         <v>Agg</v>
       </c>
       <c r="V17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L2 portfolio segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W17" t="str">
@@ -1896,7 +1896,7 @@
         <v>Agg</v>
       </c>
       <c r="Z17" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level total_cross_entity_exposure_usd per L1 business segment segment.
+        <v xml:space="preserve">Sum of cross-entity committed exposure per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA17" t="str">
@@ -1911,14 +1911,14 @@
         <v>EXP-009</v>
       </c>
       <c r="B18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Number of days outstanding payments is past due as grouped into 3 "buckets", 0-30 Days, 31-60 Days, 61-90+ Days. Used for staging classification and early credit deterioration monitoring.
+        <v xml:space="preserve">Maximum days payment overdue per facility, calculated from raw payment records in the payment_ledger table. For each facility, identifies payments where applied amount &lt; amount due, computes days overdue as reporting date minus payment_due_date, takes the MAX, then classifies into buckets: 1 = 0-30 days, 2 = 31-60 days, 3 = 61-90+ days. At aggregate levels, reports the worst (MAX) bucket across constituents.
 </v>
       </c>
       <c r="C18" t="str">
         <v>Days Payment Overdue Bucket</v>
       </c>
       <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID lookup the Payments records in the Payment Lockbox table, For each payment record where [Payment_Due_Date] &gt; Today() IF ([Pmt_Applied] &lt;[Pmt_Due])&gt;=1, THEN Today() - [Payment_due_date] ==[Days Overdue] SELECT MAX ([Days Overdue] then lookup in Payments Overdue bucket)
+        <v xml:space="preserve">For each facility, lookup payment records in payment_ledger where payment_due_date &lt; reporting date and payment_applied_amt &lt; payment_amount_due (underpaid). Calculate days overdue = reporting date minus payment_due_date. Take MAX days overdue, then classify into overdue bucket: 1 (0-30), 2 (31-60), 3 (61-90+).
 </v>
       </c>
       <c r="E18" t="str">
@@ -1937,7 +1937,7 @@
         <v>Calc</v>
       </c>
       <c r="J18" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each Facility_ID lookup the Payments records in the Payment Lockbox table, For each payment record where [Payment_Due_Date] &gt; Today() IF ([Pmt_Applied] &lt;[Pmt_Due])&gt;=1, THEN Today() - [Payment_due_date] ==[Days Overdue] SELECT MAX ([Days Overdue] then lookup in Payments Overdue bucket)
+        <v xml:space="preserve">For each facility, lookup payment records in payment_ledger where payment_due_date &lt; reporting date and payment_applied_amt &lt; payment_amount_due (underpaid). Calculate days overdue = reporting date minus payment_due_date. Take MAX days overdue, then classify into overdue bucket: 1 (0-30), 2 (31-60), 3 (61-90+).
 </v>
       </c>
       <c r="K18" t="str">
@@ -1950,7 +1950,7 @@
         <v>Agg</v>
       </c>
       <c r="N18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per counterparty.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket across all facilities per counterparty. Identifies the most severely overdue facility for each borrower.
 </v>
       </c>
       <c r="O18" t="str">
@@ -1963,7 +1963,7 @@
         <v>Agg</v>
       </c>
       <c r="R18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L3 desk segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L3 desk segment. Shows the most severe delinquency in each organizational unit.
 </v>
       </c>
       <c r="S18" t="str">
@@ -1976,7 +1976,7 @@
         <v>Agg</v>
       </c>
       <c r="V18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L2 portfolio segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W18" t="str">
@@ -1989,7 +1989,7 @@
         <v>Agg</v>
       </c>
       <c r="Z18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Worst (MAX) facility-level dpd_bucket_code per L1 business segment.
+        <v xml:space="preserve">Worst-case (MAX) overdue bucket per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA18" t="str">
@@ -2509,14 +2509,25 @@
         <v>EXP-015</v>
       </c>
       <c r="B24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Expected Loss divided by Exposure. Derived KPI measuring loss intensity relative to exposure size, enabling comparative risk ranking across facilities or counterparties.
+        <v xml:space="preserve">Expected Loss as a percentage of committed exposure. Computed from L2 atomic risk parameters: PD (probability of default) × LGD (loss given default). At aggregate levels, uses sum-ratio rollup: SUM(PD × LGD × Committed) / SUM(Committed) × 100 — the exposure-weighted average EL rate. This ensures mathematically consistent aggregation (never averages pre-computed rates). Key credit risk quantification metric for comparing loss intensity across facilities, counterparties, and business segments.
+Ingredient derivation:
+  - PD (pd_pct): L2 facility_risk_snapshot — probability of default (%)
+  - LGD (lgd_pct): L2 facility_risk_snapshot — loss given default (%)
+  - Committed Exposure (committed_amount): L2 facility_exposure_snapshot — raw
+  - EL Rate = PD × LGD (at facility level, committed cancels in ratio)
+  - Aggregate EL Rate = SUM(PD × LGD × Committed) / SUM(Committed) × 100
 </v>
       </c>
       <c r="C24" t="str">
         <v>Expected Loss Rate (%)</v>
       </c>
       <c r="D24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of expected_loss_rate_pct per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount from l2.facility_exposure_snapshot
+  3. COMPUTE EL Rate = SUM(PD/100 × LGD/100 × Committed) / SUM(Committed) × 100
+     At facility grain, committed cancels → EL Rate ≈ PD × LGD / 100
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2)
 </v>
       </c>
       <c r="E24" t="str">
@@ -2532,10 +2543,15 @@
         <v>Y</v>
       </c>
       <c r="I24" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="J24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of expected_loss_rate_pct per facility.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount from l2.facility_exposure_snapshot
+  3. COMPUTE EL Rate = SUM(PD/100 × LGD/100 × Committed) / SUM(Committed) × 100
+     At facility grain, committed cancels → EL Rate ≈ PD × LGD / 100
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2)
 </v>
       </c>
       <c r="K24" t="str">
@@ -2545,10 +2561,15 @@
         <v>Y</v>
       </c>
       <c r="M24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD pd_pct, lgd_pct for all facilities belonging to this counterparty
+  2. LOAD committed_amount for each facility
+  3. CONVERT to USD via l2.fx_rate spot rate
+  4. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup with FX: exposure-weighted average EL rate in USD terms.
 </v>
       </c>
       <c r="O24" t="str">
@@ -2558,10 +2579,14 @@
         <v>Y</v>
       </c>
       <c r="Q24" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="R24" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level expected_loss_rate_pct per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per desk.
 </v>
       </c>
       <c r="S24" t="str">
@@ -2571,10 +2596,14 @@
         <v>Y</v>
       </c>
       <c r="U24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per portfolio.
 </v>
       </c>
       <c r="W24" t="str">
@@ -2584,10 +2613,14 @@
         <v>Y</v>
       </c>
       <c r="Y24" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z24" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level expected_loss_rate_pct per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(PD × LGD × Committed × FX) / SUM(Committed × FX) × 100
+Sum-ratio rollup: exposure-weighted average EL rate per segment.
 </v>
       </c>
       <c r="AA24" t="str">
@@ -2602,14 +2635,25 @@
         <v>EXP-016</v>
       </c>
       <c r="B25" t="str" xml:space="preserve">
-        <v xml:space="preserve">PD × LGD × Exposure expressed in USD. Calculated forward-looking loss metric supporting provisioning, capital planning, and stress testing analytics.
+        <v xml:space="preserve">Expected Loss in dollar terms: PD × LGD × Committed Exposure × Bank Share. Computed from L2 atomic risk parameters and exposure data — NOT from stressed scenarios. This is the base (unstressed) expected credit loss, the foundation for provisioning, capital planning, and CECL/IFRS 9 reserve estimation.
+Ingredient derivation:
+  - PD (pd_pct): L2 facility_risk_snapshot — probability of default (%)
+  - LGD (lgd_pct): L2 facility_risk_snapshot — loss given default (%)
+  - Committed Exposure (committed_amount): L2 facility_exposure_snapshot — raw
+  - Bank Share (bank_share_pct): L2 facility_exposure_snapshot — participation %
+  - EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Rollup uses direct-sum: SUM(facility EL) at each aggregate level. FX conversion applied at aggregate levels for multi-currency portfolios.
 </v>
       </c>
       <c r="C25" t="str">
         <v>Expected Loss ($)</v>
       </c>
       <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount, bank_share_pct from l2.facility_exposure_snapshot
+  3. COMPUTE EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2), bank_share_pct (L2)
 </v>
       </c>
       <c r="E25" t="str">
@@ -2625,10 +2669,14 @@
         <v>Y</v>
       </c>
       <c r="I25" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="J25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(stressed_expected_loss) per facility from stress_test_result. Weighted by bank share percentage.
+        <v xml:space="preserve">For each facility:
+  1. LOAD pd_pct, lgd_pct from l2.facility_risk_snapshot
+  2. LOAD committed_amount, bank_share_pct from l2.facility_exposure_snapshot
+  3. COMPUTE EL = (PD/100) × (LGD/100) × Committed × (Bank Share/100)
+Ingredients: pd_pct (L2), lgd_pct (L2), committed_amount (L2), bank_share_pct (L2)
 </v>
       </c>
       <c r="K25" t="str">
@@ -2641,7 +2689,11 @@
         <v>Agg</v>
       </c>
       <c r="N25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD facility-level EL for all facilities of this counterparty
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) = Counterparty EL (USD)
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="O25" t="str">
@@ -2654,7 +2706,11 @@
         <v>Agg</v>
       </c>
       <c r="R25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per desk
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="S25" t="str">
@@ -2667,7 +2723,11 @@
         <v>Agg</v>
       </c>
       <c r="V25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per portfolio
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="W25" t="str">
@@ -2680,7 +2740,11 @@
         <v>Agg</v>
       </c>
       <c r="Z25" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level stressed_expected_loss per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. CONVERT to USD via l2.fx_rate spot rate
+  3. COMPUTE SUM(facility EL × FX rate) per business segment
+Direct-sum rollup with FX conversion.
 </v>
       </c>
       <c r="AA25" t="str">
@@ -3927,14 +3991,15 @@
         <v>EXP-030</v>
       </c>
       <c r="B39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Model-estimated probability of default within defined horizon. Core credit risk input supporting capital modeling, expected loss estimation, stress testing, and risk appetite alignment.
+        <v xml:space="preserve">Model-estimated probability of default (PD) within the defined rating horizon. At facility level, sources the raw pd_pct from L2 facility_risk_snapshot. At aggregate levels, computes the exposure- weighted average: SUM(pd_pct × committed_amount) / SUM(committed_amount). This weighted-avg rollup avoids Simpson's paradox — never averages pre-computed PD rates. Core credit risk input supporting IRB capital modeling, expected loss estimation (EL = PD × LGD × EAD), stress testing, and risk appetite alignment.
 </v>
       </c>
       <c r="C39" t="str">
         <v>Probability of Default (%)</v>
       </c>
       <c r="D39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pd_pct from facility_risk_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Direct lookup of pd_pct from facility_risk_snapshot for each facility.
+Ingredients: pd_pct (L2 facility_risk_snapshot — raw model output)
 </v>
       </c>
       <c r="E39" t="str">
@@ -3953,7 +4018,8 @@
         <v>Raw</v>
       </c>
       <c r="J39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pd_pct from facility_risk_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Direct lookup of pd_pct from facility_risk_snapshot for each facility.
+Ingredients: pd_pct (L2 facility_risk_snapshot — raw model output)
 </v>
       </c>
       <c r="K39" t="str">
@@ -3963,10 +4029,15 @@
         <v>Y</v>
       </c>
       <c r="M39" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="N39" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pd_pct per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD pd_pct and committed_amount per facility
+  2. COMPUTE exposure-weighted average PD:
+     SUM(pd_pct × committed_amount) / SUM(committed_amount)
+Weighted-avg rollup ensures large-exposure facilities dominate the
+counterparty-level PD, avoiding equal-weight averaging bias.
 </v>
       </c>
       <c r="O39" t="str">
@@ -3979,7 +4050,11 @@
         <v>Avg</v>
       </c>
       <c r="R39" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level pd_pct per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOAD pd_pct and committed_amount per facility
+  2. JOIN l1.enterprise_business_taxonomy on lob_segment_id
+  3. COMPUTE SUM(pd_pct × committed_amount) / SUM(committed_amount)
+Weighted-avg rollup per desk.
 </v>
       </c>
       <c r="S39" t="str">
@@ -3992,7 +4067,11 @@
         <v>Avg</v>
       </c>
       <c r="V39" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level pd_pct per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE SUM(pd_pct × committed_amount) / SUM(committed_amount)
+Weighted-avg rollup per portfolio. Per spec:
+Σ(probability_of_default × Outstanding_Exposure) / Σ(Total Committed Amount)
 </v>
       </c>
       <c r="W39" t="str">
@@ -4002,10 +4081,13 @@
         <v>Y</v>
       </c>
       <c r="Y39" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="Z39" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pd_pct per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE SUM(pd_pct × committed_amount) / SUM(committed_amount)
+Weighted-avg rollup per business segment.
 </v>
       </c>
       <c r="AA39" t="str">
@@ -5796,14 +5878,15 @@
         <v>PRC-003</v>
       </c>
       <c r="B59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of exposures within portfolio with approved pricing or policy exceptions. Derived governance KPI measuring policy discipline and risk culture strength.
+        <v xml:space="preserve">Percentage of facilities with approved pricing or policy exceptions. Computed as COUNT(exception facilities) / COUNT(total facilities) × 100. Sourced from L2 facility_pricing_snapshot — the atomic pricing record — using the is_pricing_exception_flag. At aggregate levels, uses count-ratio rollup: re-counts exceptions and totals across all constituent facilities, never averages pre-computed rates. Key governance KPI measuring policy discipline, risk culture strength, and pricing override frequency.
 </v>
       </c>
       <c r="C59" t="str">
         <v>Exception Rate (%)</v>
       </c>
       <c r="D59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if pricing exception, 0 otherwise.
+        <v xml:space="preserve">Binary flag: 1.0 if pricing exception approved, 0.0 otherwise.
+Ingredients: is_pricing_exception_flag (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="E59" t="str">
@@ -5822,7 +5905,8 @@
         <v>Calc</v>
       </c>
       <c r="J59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Binary flag: 1 if pricing exception, 0 otherwise.
+        <v xml:space="preserve">Binary flag: 1.0 if pricing exception approved, 0.0 otherwise.
+Ingredients: is_pricing_exception_flag (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="K59" t="str">
@@ -5835,7 +5919,10 @@
         <v>Calc</v>
       </c>
       <c r="N59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD is_pricing_exception_flag for all facilities of this counterparty
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup: re-counts from facility-level flags.
 </v>
       </c>
       <c r="O59" t="str">
@@ -5848,7 +5935,10 @@
         <v>Calc</v>
       </c>
       <c r="R59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L3 desk.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOOKUP managed_segment_id from enterprise_business_taxonomy
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per desk.
 </v>
       </c>
       <c r="S59" t="str">
@@ -5861,7 +5951,10 @@
         <v>Calc</v>
       </c>
       <c r="V59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L2 portfolio.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per portfolio.
 </v>
       </c>
       <c r="W59" t="str">
@@ -5874,7 +5967,10 @@
         <v>Calc</v>
       </c>
       <c r="Z59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Percentage of facilities with pricing exception per L1 business segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per business segment.
 </v>
       </c>
       <c r="AA59" t="str">
@@ -6075,14 +6171,18 @@
         <v>PRC-006</v>
       </c>
       <c r="B62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Pricing classification tier assigned to facility. Supports structured pricing strategy and yield segmentation.
+        <v xml:space="preserve">Pricing classification tier derived by range-joining the facility's spread (spread_bps from L2 facility_pricing_snapshot) against the pricing_tier_dim reference table (spread_min_bps/spread_max_bps). Returns the tier_ordinal at facility level and at aggregate levels classifies the exposure-weighted average spread into the corresponding tier. Supports pricing strategy segmentation, yield curve analysis, and risk-adjusted return monitoring.
 </v>
       </c>
       <c r="C62" t="str">
         <v>Pricing Tier</v>
       </c>
       <c r="D62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier_code from facility_detail_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">For each facility:
+  1. LOAD spread_bps from l2.facility_pricing_snapshot
+  2. RANGE-JOIN against l1.pricing_tier_dim
+     WHERE spread_bps &gt;= spread_min_bps AND spread_bps &lt; spread_max_bps
+  3. RETURN tier_ordinal — the numeric tier classification
 </v>
       </c>
       <c r="E62" t="str">
@@ -6098,10 +6198,14 @@
         <v>Y</v>
       </c>
       <c r="I62" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="J62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier_code from facility_detail_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">For each facility:
+  1. LOAD spread_bps from l2.facility_pricing_snapshot
+  2. RANGE-JOIN against l1.pricing_tier_dim
+     WHERE spread_bps &gt;= spread_min_bps AND spread_bps &lt; spread_max_bps
+  3. RETURN tier_ordinal — the numeric tier classification
 </v>
       </c>
       <c r="K62" t="str">
@@ -6111,10 +6215,15 @@
         <v>Y</v>
       </c>
       <c r="M62" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="N62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read pricing_tier_code per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD spread_bps and committed_amount per facility
+  2. COMPUTE weighted average spread:
+     SUM(spread_bps × committed_amount) / SUM(committed_amount)
+  3. RANGE-JOIN weighted avg spread against l1.pricing_tier_dim
+  4. RETURN tier_ordinal for the counterparty's blended spread
 </v>
       </c>
       <c r="O62" t="str">
@@ -6124,10 +6233,13 @@
         <v>Y</v>
       </c>
       <c r="Q62" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R62" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. Compute exposure-weighted average spread across desk facilities
+  2. Classify against pricing_tier_dim ranges
+  3. RETURN tier_ordinal for the desk's blended spread
 </v>
       </c>
       <c r="S62" t="str">
@@ -6137,10 +6249,13 @@
         <v>Y</v>
       </c>
       <c r="U62" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V62" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. Compute exposure-weighted average spread
+  3. Classify against pricing_tier_dim ranges
 </v>
       </c>
       <c r="W62" t="str">
@@ -6150,10 +6265,13 @@
         <v>Y</v>
       </c>
       <c r="Y62" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z62" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_tier_code per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. Compute exposure-weighted average spread
+  3. Classify against pricing_tier_dim ranges
 </v>
       </c>
       <c r="AA62" t="str">
@@ -6354,14 +6472,16 @@
         <v>PRC-009</v>
       </c>
       <c r="B65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Boolean indicator identifying whether the exposure was approved outside standard pricing policy thresholds at origination or amendment.
+        <v xml:space="preserve">Pricing exception effectiveness metric. At facility level, returns an ordinal encoding of the pricing_exception_status (APPROVED=3, PENDING=2, DENIED=1, NONE=0). At aggregate levels, computes the exception rate as COUNT(exception facilities) / COUNT(total facilities) × 100, following the count-ratio rollup pattern. Re-counts at each level to avoid Simpson's paradox. Complements PRC-003 (Exception Rate) with status-level detail for governance drill-down.
 </v>
       </c>
       <c r="C65" t="str">
-        <v>Pricing Exception Flag (Y/N)</v>
+        <v>Pricing Exception Status</v>
       </c>
       <c r="D65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated pricing_exception_flag per facility.
+        <v xml:space="preserve">Ordinal encoding of pricing_exception_status per facility:
+  APPROVED = 3, PENDING = 2, DENIED = 1, NONE/NULL = 0.
+Ingredients: pricing_exception_status (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="E65" t="str">
@@ -6380,63 +6500,79 @@
         <v>Calc</v>
       </c>
       <c r="J65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated pricing_exception_flag per facility.
+        <v xml:space="preserve">Ordinal encoding of pricing_exception_status per facility:
+  APPROVED = 3, PENDING = 2, DENIED = 1, NONE/NULL = 0.
+Ingredients: pricing_exception_status (L2 facility_pricing_snapshot)
 </v>
       </c>
       <c r="K65" t="str">
-        <v>Pricing Exception Flag (Y/N) (facility)</v>
+        <v>Pricing Exception Status (facility)</v>
       </c>
       <c r="L65" t="str">
         <v>Y</v>
       </c>
       <c r="M65" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N65" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_exception_flag per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD is_pricing_exception_flag for all facilities
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup: re-counts from facility-level flags.
 </v>
       </c>
       <c r="O65" t="str">
-        <v>Pricing Exception Flag (Y/N) (counterparty)</v>
+        <v>Pricing Exception Status (counterparty)</v>
       </c>
       <c r="P65" t="str">
         <v>Y</v>
       </c>
       <c r="Q65" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R65" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_exception_flag per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. JOIN l1.enterprise_business_taxonomy on lob_segment_id
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per desk.
 </v>
       </c>
       <c r="S65" t="str">
-        <v>Pricing Exception Flag (Y/N) (desk)</v>
+        <v>Pricing Exception Status (desk)</v>
       </c>
       <c r="T65" t="str">
         <v>Y</v>
       </c>
       <c r="U65" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V65" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_exception_flag per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per portfolio. Drill-down returns exception
+facility details: Facility_ID, Facility_Name, Counterparty_ID,
+Counterparty_Name, Exception_Status, All_in_Rate.
 </v>
       </c>
       <c r="W65" t="str">
-        <v>Pricing Exception Flag (Y/N) (portfolio)</v>
+        <v>Pricing Exception Status (portfolio)</v>
       </c>
       <c r="X65" t="str">
         <v>Y</v>
       </c>
       <c r="Y65" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z65" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level pricing_exception_flag per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE COUNT(exceptions) / COUNT(total facilities) × 100
+Count-ratio rollup per business segment.
 </v>
       </c>
       <c r="AA65" t="str">
-        <v>Pricing Exception Flag (Y/N) (business_segment)</v>
+        <v>Pricing Exception Status (business_segment)</v>
       </c>
       <c r="AB65" t="str">
         <v/>
@@ -6830,14 +6966,14 @@
         <v>REF-004</v>
       </c>
       <c r="B70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Unique system identifier assigned to the borrower or obligor. Used for exposure aggregation and risk consolidation.
+        <v xml:space="preserve">Unique system identifier assigned to the borrower or obligor. Used for exposure aggregation and risk consolidation across the GSIB. At facility level, returns the counterparty_id linked to each facility. At upper levels, returns COUNT(DISTINCT counterparty_id) — the number of unique obligors in each organizational segment.
 </v>
       </c>
       <c r="C70" t="str">
         <v>Counterparty ID</v>
       </c>
       <c r="D70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="E70" t="str">
@@ -6856,7 +6992,7 @@
         <v>Raw</v>
       </c>
       <c r="J70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each active facility. Uses current records only (SCD2 filtered).
 </v>
       </c>
       <c r="K70" t="str">
@@ -6869,7 +7005,7 @@
         <v>Raw</v>
       </c>
       <c r="N70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Identity — returns counterparty_id for each current counterparty.
 </v>
       </c>
       <c r="O70" t="str">
@@ -6882,7 +7018,7 @@
         <v>Agg</v>
       </c>
       <c r="R70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L3 desk segment — number of unique obligors in each desk.
 </v>
       </c>
       <c r="S70" t="str">
@@ -6895,7 +7031,7 @@
         <v>Agg</v>
       </c>
       <c r="V70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L2 portfolio segment — number of unique obligors in each portfolio.
 </v>
       </c>
       <c r="W70" t="str">
@@ -6908,7 +7044,7 @@
         <v>Agg</v>
       </c>
       <c r="Z70" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L1 business segment segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L1 business segment — number of unique obligors in each business segment.
 </v>
       </c>
       <c r="AA70" t="str">
@@ -6923,14 +7059,14 @@
         <v>REF-005</v>
       </c>
       <c r="B71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Descriptive name of the counterparty as documented in the credit agreement. Used for reporting clarity and operational reference.
+        <v xml:space="preserve">Legal name of the counterparty as documented in the credit agreement. At facility level, returns the counterparty_id (numeric proxy for the name since metric values are numeric). At counterparty level, identity lookup. At upper levels, COUNT(DISTINCT counterparty_id) — number of unique named obligors per organizational segment. Used for reporting clarity and operational reference across all regulatory submissions.
 </v>
       </c>
       <c r="C71" t="str">
         <v>Counterparty Name</v>
       </c>
       <c r="D71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_name from counterparty for each facility's counterparty.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="E71" t="str">
@@ -6949,7 +7085,7 @@
         <v>Raw</v>
       </c>
       <c r="J71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_name from counterparty for each facility's counterparty.
+        <v xml:space="preserve">Lookup counterparty_id from facility_master for each active facility. The numeric counterparty_id serves as proxy for the legal name (string values resolved via counterparty dimension join at display time). Uses current records only.
 </v>
       </c>
       <c r="K71" t="str">
@@ -6959,10 +7095,10 @@
         <v>Y</v>
       </c>
       <c r="M71" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="N71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per counterparty.
+        <v xml:space="preserve">Identity — returns counterparty_id for each current counterparty. Legal name resolved via counterparty dimension join at display time.
 </v>
       </c>
       <c r="O71" t="str">
@@ -6975,7 +7111,7 @@
         <v>Agg</v>
       </c>
       <c r="R71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L3 desk segment — number of unique named obligors in each desk.
 </v>
       </c>
       <c r="S71" t="str">
@@ -6988,7 +7124,7 @@
         <v>Agg</v>
       </c>
       <c r="V71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L2 portfolio segment — number of unique named obligors in each portfolio.
 </v>
       </c>
       <c r="W71" t="str">
@@ -7001,7 +7137,7 @@
         <v>Agg</v>
       </c>
       <c r="Z71" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with counterparty name per L1 business segment.
+        <v xml:space="preserve">COUNT(DISTINCT counterparty_id) per L1 business segment — number of unique named obligors in each business segment.
 </v>
       </c>
       <c r="AA71" t="str">
@@ -7016,14 +7152,14 @@
         <v>REF-006</v>
       </c>
       <c r="B72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Country of risk or booking location. Supports geographic concentration and sovereign risk analysis.
+        <v xml:space="preserve">Country of risk derived from the counterparty's domicile. At facility level, returns a numeric country identifier (via counterparty → country_dim join path). At counterparty level, identity lookup. At desk/portfolio/segment levels, COUNT(DISTINCT country_code) — geographic diversification indicator showing the number of unique countries represented. Supports FFIEC 009 Country Exposure Report and Basel III geographic concentration analysis.
 </v>
       </c>
       <c r="C72" t="str">
         <v>Country</v>
       </c>
       <c r="D72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of country_name from country_dim.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="E72" t="str">
@@ -7042,7 +7178,7 @@
         <v>Raw</v>
       </c>
       <c r="J72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of country_name from country_dim.
+        <v xml:space="preserve">Lookup country for each facility via counterparty → country_dim join path. Returns counterparty_id as numeric proxy (country_name resolved at display time via dimension join). Uses current records only.
 </v>
       </c>
       <c r="K72" t="str">
@@ -7055,7 +7191,7 @@
         <v>Raw</v>
       </c>
       <c r="N72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read country_name per counterparty.
+        <v xml:space="preserve">Lookup country for each counterparty via country_code → country_dim join. Returns counterparty_id as numeric proxy.
 </v>
       </c>
       <c r="O72" t="str">
@@ -7068,7 +7204,7 @@
         <v>Agg</v>
       </c>
       <c r="R72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L3 desk segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L3 desk segment — number of unique countries represented, a geographic diversification indicator.
 </v>
       </c>
       <c r="S72" t="str">
@@ -7081,7 +7217,7 @@
         <v>Agg</v>
       </c>
       <c r="V72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L2 portfolio segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L2 portfolio segment — number of unique countries represented in each portfolio.
 </v>
       </c>
       <c r="W72" t="str">
@@ -7094,7 +7230,7 @@
         <v>Agg</v>
       </c>
       <c r="Z72" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level country_name per L1 business segment segment.
+        <v xml:space="preserve">COUNT(DISTINCT country_code) per L1 business segment — geographic diversification at the highest organizational level.
 </v>
       </c>
       <c r="AA72" t="str">
@@ -7109,14 +7245,14 @@
         <v>REF-007</v>
       </c>
       <c r="B73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Unique identifier linking facility to governing credit agreement documentation.
+        <v xml:space="preserve">Unique identifier linking each facility to its governing credit agreement documentation. Used for contract tracking, facility-to-agreement linkage, and regulatory reporting. At counterparty level, returns count of distinct credit agreements per borrower.
 </v>
       </c>
       <c r="C73" t="str">
         <v>Credit Agreement ID</v>
       </c>
       <c r="D73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of credit_agreement_id from credit_agreement_master.
+        <v xml:space="preserve">Direct lookup of credit_agreement_id for each active facility via facility_master joined to credit_agreement_master.
 </v>
       </c>
       <c r="E73" t="str">
@@ -7135,7 +7271,7 @@
         <v>Raw</v>
       </c>
       <c r="J73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of credit_agreement_id from credit_agreement_master.
+        <v xml:space="preserve">Direct lookup of credit_agreement_id for each active facility via facility_master joined to credit_agreement_master.
 </v>
       </c>
       <c r="K73" t="str">
@@ -7145,10 +7281,10 @@
         <v>Y</v>
       </c>
       <c r="M73" t="str">
-        <v>Raw</v>
+        <v>Agg</v>
       </c>
       <c r="N73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read credit_agreement_id per counterparty.
+        <v xml:space="preserve">Count of distinct credit agreements per counterparty. Provides visibility into borrower complexity and multi-agreement relationships.
 </v>
       </c>
       <c r="O73" t="str">
@@ -7161,7 +7297,7 @@
         <v>Agg</v>
       </c>
       <c r="R73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L3 desk segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L3 desk segment via enterprise_business_taxonomy.
 </v>
       </c>
       <c r="S73" t="str">
@@ -7174,7 +7310,7 @@
         <v>Agg</v>
       </c>
       <c r="V73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L2 portfolio segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W73" t="str">
@@ -7187,7 +7323,7 @@
         <v>Agg</v>
       </c>
       <c r="Z73" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level credit_agreement_id per L1 business segment segment.
+        <v xml:space="preserve">Count of distinct credit agreements per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA73" t="str">
@@ -7295,14 +7431,15 @@
         <v>REF-009</v>
       </c>
       <c r="B75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Date on which loan or contract became legally effective.
+        <v xml:space="preserve">Facility effective date sourced from facility_master origination_date. At facility and counterparty levels, returns the raw date (or earliest vintage via MIN). At portfolio level, pivots to facility lifecycle tracking: counts inactive facilities whose origination date falls within 90 days of the reporting date, identifying the upcoming pipeline of facilities about to start ("Starting 90d"). Key for vintage analysis, portfolio seasoning, and facility pipeline monitoring.
 </v>
       </c>
       <c r="C75" t="str">
-        <v>Contract Origination Date</v>
+        <v>Facility Origination Date</v>
       </c>
       <c r="D75" t="str" xml:space="preserve">
         <v xml:space="preserve">Direct lookup of origination_date from facility_master.
+Ingredients: origination_date (L2 facility_master — raw field)
 </v>
       </c>
       <c r="E75" t="str">
@@ -7322,10 +7459,11 @@
       </c>
       <c r="J75" t="str" xml:space="preserve">
         <v xml:space="preserve">Direct lookup of origination_date from facility_master.
+Ingredients: origination_date (L2 facility_master — raw field)
 </v>
       </c>
       <c r="K75" t="str">
-        <v>Contract Origination Date (facility)</v>
+        <v>Facility Origination Date (facility)</v>
       </c>
       <c r="L75" t="str">
         <v>Y</v>
@@ -7334,11 +7472,14 @@
         <v>Agg</v>
       </c>
       <c r="N75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level origination_date) per counterparty.
+        <v xml:space="preserve">For each counterparty:
+  1. LOAD origination_date from l2.facility_master for all active facilities
+  2. COMPUTE MIN(origination_date) — earliest contract vintage
+Indicates the oldest banking relationship tenure for this counterparty.
 </v>
       </c>
       <c r="O75" t="str">
-        <v>Contract Origination Date (counterparty)</v>
+        <v>Facility Origination Date (counterparty)</v>
       </c>
       <c r="P75" t="str">
         <v>Y</v>
@@ -7347,24 +7488,33 @@
         <v>Agg</v>
       </c>
       <c r="R75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOAD origination_date from l2.facility_master
+  2. JOIN l1.enterprise_business_taxonomy on lob_segment_id
+  3. COMPUTE MIN(origination_date) — earliest vintage in desk book
 </v>
       </c>
       <c r="S75" t="str">
-        <v>Contract Origination Date (desk)</v>
+        <v>Facility Origination Date (desk)</v>
       </c>
       <c r="T75" t="str">
         <v>Y</v>
       </c>
       <c r="U75" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L2 portfolio segment.
+        <v xml:space="preserve">Facility pipeline tracking for each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. FILTER inactive facilities (is_active_flag != 'Y')
+     whose origination_date is within 90 days of current date
+  3. COMPUTE COUNT(DISTINCT facility_id) — number of upcoming facilities
+Returns the count of facilities in the "Starting (90d)" pipeline.
+Business rule: facilities not yet active with origination within ±90 days.
 </v>
       </c>
       <c r="W75" t="str">
-        <v>Contract Origination Date (portfolio)</v>
+        <v>Facility Origination Date (portfolio)</v>
       </c>
       <c r="X75" t="str">
         <v>Y</v>
@@ -7373,11 +7523,13 @@
         <v>Agg</v>
       </c>
       <c r="Z75" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level origination_date per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE MIN(origination_date) — earliest vintage in business segment
 </v>
       </c>
       <c r="AA75" t="str">
-        <v>Contract Origination Date (business_segment)</v>
+        <v>Facility Origination Date (business_segment)</v>
       </c>
       <c r="AB75" t="str">
         <v/>
@@ -8690,14 +8842,15 @@
         <v>REF-024</v>
       </c>
       <c r="B90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Identifiers of counterparties participating in the credit structures or facility as multiple-borrowers. Enables exposure attribution and concentration analysis.
+        <v xml:space="preserve">Count of distinct counterparties participating in credit structures. At counterparty level, returns the counterparty identifier directly. At desk and higher levels, counts distinct counterparties per segment to measure borrower concentration and multi-borrower facility exposure. Enables concentration analysis, relationship tracking, and syndicated deal monitoring.
 </v>
       </c>
       <c r="C90" t="str">
         <v>Participating Counterparty IDs</v>
       </c>
       <c r="D90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each facility.
+Returns the counterparty associated with the facility.
 </v>
       </c>
       <c r="E90" t="str">
@@ -8716,7 +8869,8 @@
         <v>Raw</v>
       </c>
       <c r="J90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Direct lookup of counterparty_id from facility_master for each facility.
+Returns the counterparty associated with the facility.
 </v>
       </c>
       <c r="K90" t="str">
@@ -8729,7 +8883,8 @@
         <v>Raw</v>
       </c>
       <c r="N90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of counterparty_id from counterparty.
+        <v xml:space="preserve">Identity: returns counterparty_id for each active counterparty.
+Enables direct counterparty identification in drill-down views.
 </v>
       </c>
       <c r="O90" t="str">
@@ -8739,10 +8894,14 @@
         <v>Y</v>
       </c>
       <c r="Q90" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R90" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L3 desk segment.
+        <v xml:space="preserve">For each L3 Desk segment:
+  1. LOAD all facilities from l2.facility_master
+  2. JOIN l1.enterprise_business_taxonomy on lob_segment_id
+  3. COMPUTE COUNT(DISTINCT counterparty_id) — unique borrowers per desk
+Measures borrower concentration within each desk.
 </v>
       </c>
       <c r="S90" t="str">
@@ -8752,10 +8911,12 @@
         <v>Y</v>
       </c>
       <c r="U90" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V90" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L2 portfolio segment.
+        <v xml:space="preserve">For each L2 Portfolio segment:
+  1. Walk UP hierarchy: L3 desk → L2 portfolio via parent_segment_id
+  2. COMPUTE COUNT(DISTINCT counterparty_id) — unique borrowers per portfolio
 </v>
       </c>
       <c r="W90" t="str">
@@ -8765,10 +8926,12 @@
         <v>Y</v>
       </c>
       <c r="Y90" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z90" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level counterparty_id per L1 business segment segment.
+        <v xml:space="preserve">For each L1 Business Segment / LoB:
+  1. Walk UP hierarchy: L3 → L2 → L1 via parent_segment_id chain
+  2. COMPUTE COUNT(DISTINCT counterparty_id) — unique borrowers per segment
 </v>
       </c>
       <c r="AA90" t="str">
@@ -9620,14 +9783,14 @@
         <v>RSK-001</v>
       </c>
       <c r="B100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Most recent internal credit rating assigned at reporting date. Used for segmentation and exposure-weighted risk aggregation.
+        <v xml:space="preserve">Risk rating tier derived from counterparty probability of default (PD). Each counterparty's pd_annual is matched against the risk_rating_tier_dim reference table (pd_min_pct / pd_max_pct boundaries) to assign a tier classification. At facility level, the tier is inherited from the owning counterparty. At aggregate levels, MAX (worst-case) tier ordinal is reported.
 </v>
       </c>
       <c r="C100" t="str">
         <v>Risk Rating Tier</v>
       </c>
       <c r="D100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read risk_rating_status from counterparty_rating_observation for each facility.
+        <v xml:space="preserve">For each facility, inherit the risk rating tier from the owning counterparty. Join facility_master to counterparty, then range-match counterparty pd_annual against risk_rating_tier_dim to derive the tier ordinal (display_order).
 </v>
       </c>
       <c r="E100" t="str">
@@ -9643,10 +9806,10 @@
         <v>Y</v>
       </c>
       <c r="I100" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="J100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read risk_rating_status from counterparty_rating_observation for each facility.
+        <v xml:space="preserve">For each facility, inherit the risk rating tier from the owning counterparty. Join facility_master to counterparty, then range-match counterparty pd_annual against risk_rating_tier_dim to derive the tier ordinal (display_order).
 </v>
       </c>
       <c r="K100" t="str">
@@ -9656,10 +9819,10 @@
         <v>Y</v>
       </c>
       <c r="M100" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per counterparty.
+        <v xml:space="preserve">For each counterparty, look up pd_annual and range-match against risk_rating_tier_dim where pd_annual &gt;= pd_min_pct AND pd_annual &lt; pd_max_pct. Returns the tier ordinal (display_order). Counterparties with NULL PD receive tier 0 (unrated).
 </v>
       </c>
       <c r="O100" t="str">
@@ -9672,7 +9835,7 @@
         <v>Agg</v>
       </c>
       <c r="R100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L3 desk segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal across all counterparties in the L3 desk segment. Higher ordinal = riskier tier. Full tier distribution available via counterparty-level drill-down.
 </v>
       </c>
       <c r="S100" t="str">
@@ -9685,7 +9848,7 @@
         <v>Agg</v>
       </c>
       <c r="V100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L2 portfolio segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal per L2 portfolio segment. Traverses EBT hierarchy L3 → L2 via parent_segment_id.
 </v>
       </c>
       <c r="W100" t="str">
@@ -9698,7 +9861,7 @@
         <v>Agg</v>
       </c>
       <c r="Z100" t="str" xml:space="preserve">
-        <v xml:space="preserve">COUNT of facilities with risk rating per L1 business segment.
+        <v xml:space="preserve">Worst-case (MAX) risk rating tier ordinal per L1 business segment. Full EBT hierarchy traversal L3 → L2 → L1.
 </v>
       </c>
       <c r="AA100" t="str">

</xml_diff>

<commit_message>
Regenerate Excel after merge of 5 GSIB metrics branch
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/metrics_dimensions_filled.xlsx
+++ b/data/metrics_dimensions_filled.xlsx
@@ -2766,11 +2766,21 @@
         <v>Undrawn Exposure ($)</v>
       </c>
       <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
-2. Subtract from committed_facility_amt to get unfunded amount
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
-Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY fm.facility_id
+6. COMPUTE
+   metric_value = (committed_facility_amt - SUM(funded_amount))
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="E26" t="str">
@@ -2789,11 +2799,21 @@
         <v>Calc</v>
       </c>
       <c r="J26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. SUM(funded_amount) from PRINCIPAL position_detail rows per facility
-2. Subtract from committed_facility_amt to get unfunded amount
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
-Ensures: Committed Exposure = Outstanding Exposure + Undrawn Exposure
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY fm.facility_id
+6. COMPUTE
+   metric_value = (committed_facility_amt - SUM(funded_amount))
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="K26" t="str">
@@ -2806,8 +2826,13 @@
         <v>Calc</v>
       </c>
       <c r="N26" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty, sum facility-level undrawn exposure weighted
-by participation_pct from facility_counterparty_participation.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_counterparty_participation  (fcp)
+   ON    fcp.facility_id = fac.facility_id
+   AND   fcp.is_current_flag = 'Y'
+3. GROUP BY fcp.counterparty_id
+4. COMPUTE
+   metric_value = SUM(facility_undrawn * participation_pct)
 </v>
       </c>
       <c r="O26" t="str">
@@ -2820,8 +2845,15 @@
         <v>Agg</v>
       </c>
       <c r="R26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L3 desk segment.
-Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="S26" t="str">
@@ -2834,8 +2866,16 @@
         <v>Agg</v>
       </c>
       <c r="V26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L2 portfolio segment.
-Traverses L3 -&gt; L2 via parent_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="W26" t="str">
@@ -2848,8 +2888,18 @@
         <v>Agg</v>
       </c>
       <c r="Z26" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level undrawn exposure per L1 business segment.
-Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
+        <v xml:space="preserve">1. LOAD  facility-level undrawn exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l1)
+   ON    ebt_l1.managed_segment_id = ebt_l2.parent_segment_id
+6. GROUP BY ebt_l1.managed_segment_id
+7. COMPUTE
+   metric_value = SUM(facility_undrawn)
 </v>
       </c>
       <c r="AA26" t="str">
@@ -2864,17 +2914,28 @@
         <v>EXP-018</v>
       </c>
       <c r="B27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Bank-share-adjusted funded (drawn) exposure amount. Represents the portion of committed credit currently utilized by the borrower. Maps to FR Y-14Q Field 25 (Utilized Exposure Global, MDRM G075).
+        <v xml:space="preserve">Bank-share-adjusted funded (drawn) exposure amount. Represents the portion of committed credit currently utilized by the borrower. Maps to FR Y-14Q Field 25 (Utilized Exposure Global, MDRM G075). Counterparty level uses exposure_counterparty_attribution for risk-shifted attribution weighting per Basel III requirements.
 </v>
       </c>
       <c r="C27" t="str">
         <v>Outstanding Exposure ($)</v>
       </c>
       <c r="D27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(funded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY pos.facility_id
+6. COMPUTE
+   metric_value = SUM(funded_amount)
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="E27" t="str">
@@ -2893,10 +2954,21 @@
         <v>Calc</v>
       </c>
       <c r="J27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each active facility:
-1. Join position -&gt; position_detail on position_id (both as_of_date filtered)
-2. SUM(funded_amount) across all positions for the facility
-3. Multiply by COALESCE(bank_share_pct, 100) / 100 from facility_lender_allocation
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.position_detail  (pdtl)
+   ON    pdtl.position_id = pos.position_id
+   AND   pdtl.detail_type = 'PRINCIPAL'
+3. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+4. LEFT JOIN  l2.facility_lender_allocation  (fla)
+   ON    fla.facility_id = fm.facility_id
+   AND   fla.is_current_flag = 'Y'
+5. GROUP BY pos.facility_id
+6. COMPUTE
+   metric_value = SUM(funded_amount)
+                  * COALESCE(bank_share_pct, 100) / 100
 </v>
       </c>
       <c r="K27" t="str">
@@ -2909,9 +2981,13 @@
         <v>Calc</v>
       </c>
       <c r="N27" t="str" xml:space="preserve">
-        <v xml:space="preserve">For each counterparty, sum facility-level outstanding exposure weighted
-by participation_pct from facility_counterparty_participation.
-Uses contractual pro-rata basis per FR Y-14Q requirements.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.exposure_counterparty_attribution  (eca)
+   ON    eca.facility_id = fac.facility_id
+   AND   eca.as_of_date = :as_of_date
+3. GROUP BY eca.counterparty_id
+4. COMPUTE
+   metric_value = SUM(facility_outstanding * attribution_pct)
 </v>
       </c>
       <c r="O27" t="str">
@@ -2924,8 +3000,15 @@
         <v>Agg</v>
       </c>
       <c r="R27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L3 desk segment.
-Joins facility_master.lob_segment_id to enterprise_business_taxonomy.managed_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="S27" t="str">
@@ -2938,8 +3021,16 @@
         <v>Agg</v>
       </c>
       <c r="V27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L2 portfolio segment.
-Traverses L3 -&gt; L2 via parent_segment_id.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3)
+   ON    ebt_l3.managed_segment_id = fm.lob_segment_id
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l2)
+   ON    ebt_l2.managed_segment_id = ebt_l3.parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="W27" t="str">
@@ -2952,8 +3043,14 @@
         <v>Agg</v>
       </c>
       <c r="Z27" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level outstanding exposure per L1 business segment.
-Traverses L3 -&gt; L2 -&gt; L1 via parent_segment_id chain.
+        <v xml:space="preserve">1. LOAD  facility-level outstanding exposure (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+4. GROUP BY ebt_l1.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_outstanding)
 </v>
       </c>
       <c r="AA27" t="str">
@@ -2968,14 +3065,15 @@
         <v>EXP-019</v>
       </c>
       <c r="B28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Maximum approved credit exposure authorized for the counterparty or Line of Business segment in USD. Represents formal risk appetite allocation and governance control threshold.
+        <v xml:space="preserve">Maximum approved credit exposure authorized for the counterparty or Line of Business segment in USD. Sourced directly from the limit_rule reference table. Represents formal risk appetite allocation and governance control threshold set by the Credit Risk Committee. Not applicable at individual facility level — limits are set at counterparty and organizational hierarchy levels.
 </v>
       </c>
       <c r="C28" t="str">
         <v>Exposure Limit ($)</v>
       </c>
       <c r="D28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt from lob_exposure_summary for each facility as-of reporting date.
+        <v xml:space="preserve">Not applicable — exposure limits are set at counterparty and
+organizational levels, not per individual facility. Returns NULL.
 </v>
       </c>
       <c r="E28" t="str">
@@ -2994,7 +3092,8 @@
         <v>Raw</v>
       </c>
       <c r="J28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt from lob_exposure_summary for each facility as-of reporting date.
+        <v xml:space="preserve">Not applicable — exposure limits are set at counterparty and
+organizational levels, not per individual facility. Returns NULL.
 </v>
       </c>
       <c r="K28" t="str">
@@ -3007,7 +3106,12 @@
         <v>Raw</v>
       </c>
       <c r="N28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read limit_amt per counterparty.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.counterparty_id IS NOT NULL
+2. GROUP BY lr.counterparty_id
+3. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="O28" t="str">
@@ -3017,10 +3121,18 @@
         <v>Y</v>
       </c>
       <c r="Q28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="R28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="S28" t="str">
@@ -3030,10 +3142,18 @@
         <v>Y</v>
       </c>
       <c r="U28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="V28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="W28" t="str">
@@ -3043,10 +3163,18 @@
         <v>Y</v>
       </c>
       <c r="Y28" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="Z28" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_amt per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  l1.limit_rule  (lr)
+   WHERE lr.is_current_flag = 'Y'
+   AND   lr.lob_segment_id IS NOT NULL
+2. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = lr.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+3. GROUP BY lr.lob_segment_id
+4. COMPUTE
+   metric_value = SUM(limit_amount_usd)
 </v>
       </c>
       <c r="AA28" t="str">
@@ -3061,14 +3189,25 @@
         <v>EXP-020</v>
       </c>
       <c r="B29" t="str" xml:space="preserve">
-        <v xml:space="preserve">The estimated exposure amount (in USD) expected to be outstanding if the borrower defaults.
+        <v xml:space="preserve">Estimated exposure amount outstanding if the borrower defaults, computed from L2 atomic inputs per Basel III: EAD = OB + CCF × Undrawn, where OB = drawn/funded amount, CCF = credit conversion factor from facility_risk_snapshot, and Undrawn = committed minus drawn from facility_exposure_snapshot. Bank-share adjusted via facility_exposure_snapshot. At counterparty level, weighted by participation_pct from facility_counterparty_participation per FR Y-14Q requirements.
 </v>
       </c>
       <c r="C29" t="str">
         <v>Exposure at Default ($)</v>
       </c>
       <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read exposure_at_default from credit_event_facility_link for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+   AND   frs.as_of_date = fes.as_of_date
+4. GROUP BY fes.facility_id
+5. COMPUTE
+   metric_value = (drawn_amount + CCF * undrawn_amount)
+                  * bank_share_pct / 100
 </v>
       </c>
       <c r="E29" t="str">
@@ -3084,10 +3223,21 @@
         <v>Y</v>
       </c>
       <c r="I29" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="J29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read exposure_at_default from credit_event_facility_link for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+   AND   frs.as_of_date = fes.as_of_date
+4. GROUP BY fes.facility_id
+5. COMPUTE
+   metric_value = (drawn_amount + CCF * undrawn_amount)
+                  * bank_share_pct / 100
 </v>
       </c>
       <c r="K29" t="str">
@@ -3097,10 +3247,22 @@
         <v>Y</v>
       </c>
       <c r="M29" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per counterparty.
+        <v xml:space="preserve">1. LOAD  l2.facility_exposure_snapshot  (fes)
+   WHERE fes.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fes.facility_id
+3. LEFT JOIN  l2.facility_risk_snapshot  (frs)
+   ON    frs.facility_id = fes.facility_id
+4. JOIN  l2.facility_counterparty_participation  (fcp)
+   ON    fcp.facility_id = fes.facility_id
+   AND   fcp.is_current_flag = 'Y'
+5. GROUP BY fcp.counterparty_id
+6. COMPUTE
+   metric_value = SUM((drawn + CCF * undrawn) * bank_share / 100
+                  * participation_pct)
 </v>
       </c>
       <c r="O29" t="str">
@@ -3113,7 +3275,15 @@
         <v>Agg</v>
       </c>
       <c r="R29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = fac.facility_id
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+   AND   ebt.is_current_flag = 'Y'
+4. GROUP BY ebt.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="S29" t="str">
@@ -3126,7 +3296,13 @@
         <v>Agg</v>
       </c>
       <c r="V29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2)
+   Traverse L3 -&gt; L2 via parent_segment_id
+4. GROUP BY ebt_l2.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="W29" t="str">
@@ -3139,7 +3315,13 @@
         <v>Agg</v>
       </c>
       <c r="Z29" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level exposure_at_default per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  facility-level EAD (subquery)
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+4. GROUP BY ebt_l1.managed_segment_id
+5. COMPUTE
+   metric_value = SUM(facility_ead)
 </v>
       </c>
       <c r="AA29" t="str">
@@ -3154,14 +3336,14 @@
         <v>EXP-021</v>
       </c>
       <c r="B30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Derived categorical classification (Sufficient, Approaching, Fully Utilized) of utilization level based on current drawn exposure relative to committed amount. Operational KPI providing early warning insight into limit pressure, liquidity usage, and potential capacity constraints.
+        <v xml:space="preserve">Derived categorical classification of utilization level based on current drawn exposure relative to committed amount. Maps facility utilization percentage against l1.utilization_status_dim threshold ranges to return status labels (e.g., Sufficient, Approaching, Fully Utilized). Operational KPI providing early warning insight into limit pressure, liquidity usage, and potential capacity constraints.
 </v>
       </c>
       <c r="C30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure)</v>
       </c>
       <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated utilization_status_code per facility.
+        <v xml:space="preserve">For each facility, compute utilization_pct from L2 atomic data (drawn_amount / committed_amount * 100), then match against l1.utilization_status_dim threshold ranges (utilization_min_pct &lt;= pct &lt; utilization_max_pct) to return status_name.
 </v>
       </c>
       <c r="E30" t="str">
@@ -3180,63 +3362,63 @@
         <v>Calc</v>
       </c>
       <c r="J30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated utilization_status_code per facility.
+        <v xml:space="preserve">For each facility, compute utilization_pct from L2 atomic data (drawn_amount / committed_amount * 100), then match against l1.utilization_status_dim threshold ranges (utilization_min_pct &lt;= pct &lt; utilization_max_pct) to return status_name.
 </v>
       </c>
       <c r="K30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized) (facility)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure) (facility)</v>
       </c>
       <c r="L30" t="str">
         <v>Y</v>
       </c>
       <c r="M30" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N30" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level utilization_status_code) per counterparty.
+        <v xml:space="preserve">Compute counterparty-level utilization pct via sum-ratio with FX conversion: SUM(drawn * fx) / SUM(committed * fx) * 100. Then look up status from utilization_status_dim threshold ranges.
 </v>
       </c>
       <c r="O30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized) (counterparty)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure) (counterparty)</v>
       </c>
       <c r="P30" t="str">
         <v>Y</v>
       </c>
       <c r="Q30" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R30" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level utilization_status_code per L3 desk segment.
+        <v xml:space="preserve">Compute L3 desk-level utilization pct via sum-ratio with FX conversion, then look up status from utilization_status_dim threshold ranges.
 </v>
       </c>
       <c r="S30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized) (desk)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure) (desk)</v>
       </c>
       <c r="T30" t="str">
         <v>Y</v>
       </c>
       <c r="U30" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V30" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level utilization_status_code per L2 portfolio segment.
+        <v xml:space="preserve">Compute L2 portfolio-level utilization pct via sum-ratio with FX conversion (one-hop EBT hierarchy), then look up status from utilization_status_dim threshold ranges.
 </v>
       </c>
       <c r="W30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized) (portfolio)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure) (portfolio)</v>
       </c>
       <c r="X30" t="str">
         <v>Y</v>
       </c>
       <c r="Y30" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z30" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level utilization_status_code per L1 business segment segment.
+        <v xml:space="preserve">Compute L1 business segment-level utilization pct via sum-ratio with FX conversion (two-hop EBT hierarchy), then look up status from utilization_status_dim threshold ranges.
 </v>
       </c>
       <c r="AA30" t="str">
-        <v>Facility Utilization Status (e.g., Sufficient, Approaching, Fully Utilized) (business_segment)</v>
+        <v>Utilization Status (Utilized Exposure to Committed Exposure) (business_segment)</v>
       </c>
       <c r="AB30" t="str">
         <v/>
@@ -3340,14 +3522,14 @@
         <v>EXP-023</v>
       </c>
       <c r="B32" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure × LGD expressed in dollar terms weighted based on facility-level exposure. Derived loss severity metric estimating expected recovery-adjusted loss magnitude.
+        <v xml:space="preserve">Expected dollar loss given default. Computed as EAD (drawn amount, bank share) multiplied by LGD percentage from facility risk snapshot. Expressed in local currency at facility level and FX-converted to USD at aggregate levels. Quantifies loss severity per facility and across rollup hierarchy.
 </v>
       </c>
       <c r="C32" t="str">
         <v>Loss Given Default ($)</v>
       </c>
       <c r="D32" t="str" xml:space="preserve">
-        <v xml:space="preserve">EAD * LGD (in Percentage) for all facilities across Counterparties
+        <v xml:space="preserve">EAD (bank share) x LGD% per facility in local currency.
 </v>
       </c>
       <c r="E32" t="str">
@@ -3366,7 +3548,7 @@
         <v>Calc</v>
       </c>
       <c r="J32" t="str" xml:space="preserve">
-        <v xml:space="preserve">EAD * LGD (in Percentage) for all facilities across Counterparties
+        <v xml:space="preserve">EAD (bank share) x LGD% per facility in local currency.
 </v>
       </c>
       <c r="K32" t="str">
@@ -3379,7 +3561,7 @@
         <v>Agg</v>
       </c>
       <c r="N32" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level lgd_estimate per counterparty.
+        <v xml:space="preserve">SUM of facility-level LGD$ per counterparty, FX-converted to USD.
 </v>
       </c>
       <c r="O32" t="str">
@@ -3392,7 +3574,7 @@
         <v>Agg</v>
       </c>
       <c r="R32" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level lgd_estimate per L3 desk segment.
+        <v xml:space="preserve">SUM of facility-level LGD$ per L3 desk segment, FX-converted to USD.
 </v>
       </c>
       <c r="S32" t="str">
@@ -3405,7 +3587,7 @@
         <v>Agg</v>
       </c>
       <c r="V32" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level lgd_estimate per L2 portfolio segment.
+        <v xml:space="preserve">SUM of facility-level LGD$ per L2 portfolio segment, FX-converted to USD.
 </v>
       </c>
       <c r="W32" t="str">
@@ -3418,7 +3600,7 @@
         <v>Agg</v>
       </c>
       <c r="Z32" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level lgd_estimate per L1 business segment segment.
+        <v xml:space="preserve">SUM of facility-level LGD$ per L1 business segment, FX-converted to USD.
 </v>
       </c>
       <c r="AA32" t="str">
@@ -3433,14 +3615,14 @@
         <v>EXP-024</v>
       </c>
       <c r="B33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Status of credit limit (Active, Warning, Breach). Used to monitor risk appetite breaches and exposure governance compliance.
+        <v xml:space="preserve">Utilization-based limit compliance status. At facility level reads the pre-computed limit_status_code. At aggregate levels computes drawn-to- committed utilization percentage (FX-converted to USD) and maps to a status code via utilization_status_dim thresholds. Used for credit limit monitoring and risk appetite breach detection.
 </v>
       </c>
       <c r="C33" t="str">
         <v>Limit Status</v>
       </c>
       <c r="D33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated limit_status_code per facility.
+        <v xml:space="preserve">Read pre-computed limit_status_code from facility_exposure_snapshot.
 </v>
       </c>
       <c r="E33" t="str">
@@ -3456,10 +3638,10 @@
         <v>Y</v>
       </c>
       <c r="I33" t="str">
-        <v>Calc</v>
+        <v>Raw</v>
       </c>
       <c r="J33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Calculated limit_status_code per facility.
+        <v xml:space="preserve">Read pre-computed limit_status_code from facility_exposure_snapshot.
 </v>
       </c>
       <c r="K33" t="str">
@@ -3469,10 +3651,10 @@
         <v>Y</v>
       </c>
       <c r="M33" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="N33" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_status_code per counterparty.
+        <v xml:space="preserve">Compute drawn-to-committed utilization % per counterparty (FX-converted), then map to status via utilization_status_dim thresholds.
 </v>
       </c>
       <c r="O33" t="str">
@@ -3482,10 +3664,10 @@
         <v>Y</v>
       </c>
       <c r="Q33" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R33" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_status_code per L3 desk segment.
+        <v xml:space="preserve">Compute drawn-to-committed utilization % per L3 desk segment (FX-converted), then map to status via utilization_status_dim.
 </v>
       </c>
       <c r="S33" t="str">
@@ -3495,10 +3677,10 @@
         <v>Y</v>
       </c>
       <c r="U33" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V33" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_status_code per L2 portfolio segment.
+        <v xml:space="preserve">Compute drawn-to-committed utilization % per L2 portfolio segment (FX-converted), then map to status via utilization_status_dim.
 </v>
       </c>
       <c r="W33" t="str">
@@ -3508,10 +3690,10 @@
         <v>Y</v>
       </c>
       <c r="Y33" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z33" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level limit_status_code per L1 business segment segment.
+        <v xml:space="preserve">Compute drawn-to-committed utilization % per L1 business segment (FX-converted), then map to status via utilization_status_dim.
 </v>
       </c>
       <c r="AA33" t="str">
@@ -5967,14 +6149,14 @@
         <v>PRC-004</v>
       </c>
       <c r="B60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Fee percentage applied to committed or undrawn exposure. Calculated KPI supporting pricing adequacy and revenue optimization analysis.
+        <v xml:space="preserve">Fee percentage applied to committed or undrawn exposure. Sourced from l2.facility_pricing_snapshot at facility level. Supports pricing adequacy and revenue optimization analysis. Aggregate levels use exposure-weighted average with FX conversion to USD.
 </v>
       </c>
       <c r="C60" t="str">
         <v>Fee Rate (%)</v>
       </c>
       <c r="D60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Fee Income / Average Balance
+        <v xml:space="preserve">Direct lookup of fee_rate_pct from l2.facility_pricing_snapshot.
 </v>
       </c>
       <c r="E60" t="str">
@@ -5990,10 +6172,10 @@
         <v>Y</v>
       </c>
       <c r="I60" t="str">
-        <v>Calc</v>
+        <v>Raw</v>
       </c>
       <c r="J60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Fee Income / Average Balance
+        <v xml:space="preserve">Direct lookup of fee_rate_pct from l2.facility_pricing_snapshot.
 </v>
       </c>
       <c r="K60" t="str">
@@ -6006,7 +6188,7 @@
         <v>Avg</v>
       </c>
       <c r="N60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Exposure-weighted average of fee_rate_pct across counterparty facilities.
+        <v xml:space="preserve">Supplementary (not in primary specification at counterparty level). Exposure-weighted average fee rate per counterparty with FX conversion: SUM(fee_rate * committed_amt * fx) / SUM(committed_amt * fx).
 </v>
       </c>
       <c r="O60" t="str">
@@ -6019,7 +6201,7 @@
         <v>Avg</v>
       </c>
       <c r="R60" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level fee_rate_pct per L3 desk segment.
+        <v xml:space="preserve">Supplementary. Exposure-weighted average fee rate per L3 desk segment with FX conversion.
 </v>
       </c>
       <c r="S60" t="str">
@@ -6032,7 +6214,7 @@
         <v>Avg</v>
       </c>
       <c r="V60" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level fee_rate_pct per L2 portfolio segment.
+        <v xml:space="preserve">Supplementary. Exposure-weighted average fee rate per L2 portfolio segment with FX conversion.
 </v>
       </c>
       <c r="W60" t="str">
@@ -6042,10 +6224,10 @@
         <v>Y</v>
       </c>
       <c r="Y60" t="str">
-        <v>Agg</v>
+        <v>Avg</v>
       </c>
       <c r="Z60" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level fee_rate_pct per L1 business segment segment.
+        <v xml:space="preserve">Supplementary. Exposure-weighted average fee rate per L1 business segment with FX conversion.
 </v>
       </c>
       <c r="AA60" t="str">
@@ -7517,7 +7699,7 @@
         <v>Raw</v>
       </c>
       <c r="N76" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read facility_id per counterparty.
+        <v xml:space="preserve">Representative facility_id per counterparty (MIN).
 </v>
       </c>
       <c r="O76" t="str">
@@ -7527,10 +7709,10 @@
         <v>Y</v>
       </c>
       <c r="Q76" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="R76" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_id per L3 desk segment.
+        <v xml:space="preserve">Representative facility_id per L3 desk segment (MIN).
 </v>
       </c>
       <c r="S76" t="str">
@@ -7540,10 +7722,10 @@
         <v>Y</v>
       </c>
       <c r="U76" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="V76" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_id per L2 portfolio segment.
+        <v xml:space="preserve">Representative facility_id per L2 portfolio segment (MIN).
 </v>
       </c>
       <c r="W76" t="str">
@@ -7553,10 +7735,10 @@
         <v>Y</v>
       </c>
       <c r="Y76" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="Z76" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_id per L1 business segment segment.
+        <v xml:space="preserve">Representative facility_id per L1 business segment (MIN).
 </v>
       </c>
       <c r="AA76" t="str">
@@ -7610,7 +7792,7 @@
         <v>Raw</v>
       </c>
       <c r="N77" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read facility_name per counterparty.
+        <v xml:space="preserve">Representative facility_name per counterparty (MIN alphabetical).
 </v>
       </c>
       <c r="O77" t="str">
@@ -7620,10 +7802,10 @@
         <v>Y</v>
       </c>
       <c r="Q77" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="R77" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_name per L3 desk segment.
+        <v xml:space="preserve">Representative facility_name per L3 desk segment (MIN alphabetical).
 </v>
       </c>
       <c r="S77" t="str">
@@ -7633,10 +7815,10 @@
         <v>Y</v>
       </c>
       <c r="U77" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="V77" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_name per L2 portfolio segment.
+        <v xml:space="preserve">Representative facility_name per L2 portfolio segment (MIN alphabetical).
 </v>
       </c>
       <c r="W77" t="str">
@@ -7646,10 +7828,10 @@
         <v>Y</v>
       </c>
       <c r="Y77" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="Z77" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_name per L1 business segment segment.
+        <v xml:space="preserve">Representative facility_name per L1 business segment (MIN alphabetical).
 </v>
       </c>
       <c r="AA77" t="str">
@@ -7664,14 +7846,14 @@
         <v>REF-012</v>
       </c>
       <c r="B78" t="str" xml:space="preserve">
-        <v xml:space="preserve">Type of credit facility (e.g., Term Loan, Revolver, Letter of Credit). Enables product-level segmentation, risk concentration analysis, and performance benchmarking.
+        <v xml:space="preserve">Type of credit facility (e.g., Term Loan, Revolver, Letter of Credit). Enables product-level segmentation, risk concentration analysis, and performance benchmarking. At facility level returns the facility type string; at aggregate levels returns the count of distinct active facilities in the segment for distribution analysis.
 </v>
       </c>
       <c r="C78" t="str">
         <v>Facility Type</v>
       </c>
       <c r="D78" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read facility_type from facility_exposure_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Direct lookup of facility_type from facility_master.
 </v>
       </c>
       <c r="E78" t="str">
@@ -7690,7 +7872,7 @@
         <v>Raw</v>
       </c>
       <c r="J78" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read facility_type from facility_exposure_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Direct lookup of facility_type from facility_master.
 </v>
       </c>
       <c r="K78" t="str">
@@ -7700,10 +7882,10 @@
         <v>Y</v>
       </c>
       <c r="M78" t="str">
-        <v>Agg</v>
+        <v>Raw</v>
       </c>
       <c r="N78" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM(facility-level facility_type) per counterparty.
+        <v xml:space="preserve">Not in primary specification at counterparty level. Supplementary: representative facility_type per counterparty (MIN).
 </v>
       </c>
       <c r="O78" t="str">
@@ -7716,7 +7898,7 @@
         <v>Agg</v>
       </c>
       <c r="R78" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_type per L3 desk segment.
+        <v xml:space="preserve">Count distinct active facilities per L3 desk segment. Provides facility distribution for product mix analysis.
 </v>
       </c>
       <c r="S78" t="str">
@@ -7729,7 +7911,7 @@
         <v>Agg</v>
       </c>
       <c r="V78" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_type per L2 portfolio segment.
+        <v xml:space="preserve">Count distinct active facilities per L2 portfolio segment. Provides facility distribution for product mix analysis.
 </v>
       </c>
       <c r="W78" t="str">
@@ -7742,7 +7924,7 @@
         <v>Agg</v>
       </c>
       <c r="Z78" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level facility_type per L1 business segment segment.
+        <v xml:space="preserve">Count distinct active facilities per L1 business segment. Provides facility distribution for product mix analysis.
 </v>
       </c>
       <c r="AA78" t="str">
@@ -8036,14 +8218,14 @@
         <v>REF-016</v>
       </c>
       <c r="B82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Legal entity booking or owning the exposure. Critical for regulatory capital and entity-level reporting.
+        <v xml:space="preserve">Booking legal entity for each facility exposure. At facility level returns the entity name from the legal_entity table. At aggregate levels returns the count of distinct booking entities for risk concentration analysis.
 </v>
       </c>
       <c r="C82" t="str">
         <v>Legal Entity</v>
       </c>
       <c r="D82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of legal_name from counterparty.
+        <v xml:space="preserve">Lookup legal_entity_name from legal_entity table via facility_exposure_snapshot.legal_entity_id.
 </v>
       </c>
       <c r="E82" t="str">
@@ -8062,7 +8244,7 @@
         <v>Raw</v>
       </c>
       <c r="J82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of legal_name from counterparty.
+        <v xml:space="preserve">Lookup legal_entity_name from legal_entity table via facility_exposure_snapshot.legal_entity_id.
 </v>
       </c>
       <c r="K82" t="str">
@@ -8072,10 +8254,10 @@
         <v>Y</v>
       </c>
       <c r="M82" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="N82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Direct lookup of legal_name from counterparty.
+        <v xml:space="preserve">Count of distinct booking legal entities per counterparty.
 </v>
       </c>
       <c r="O82" t="str">
@@ -8085,10 +8267,10 @@
         <v>Y</v>
       </c>
       <c r="Q82" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R82" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_name per L3 desk segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L3 desk segment.
 </v>
       </c>
       <c r="S82" t="str">
@@ -8098,10 +8280,10 @@
         <v>Y</v>
       </c>
       <c r="U82" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V82" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_name per L2 portfolio segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L2 portfolio segment.
 </v>
       </c>
       <c r="W82" t="str">
@@ -8111,10 +8293,10 @@
         <v>Y</v>
       </c>
       <c r="Y82" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z82" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_name per L1 business segment segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L1 business segment.
 </v>
       </c>
       <c r="AA82" t="str">
@@ -8129,14 +8311,14 @@
         <v>REF-017</v>
       </c>
       <c r="B83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Unique identifier assigned to legal entity in enterprise systems.
+        <v xml:space="preserve">Unique identifier for the booking legal entity. At facility level returns the entity ID. At aggregate levels returns count of distinct booking entities for entity concentration tracking.
 </v>
       </c>
       <c r="C83" t="str">
         <v>Legal Entity ID</v>
       </c>
       <c r="D83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_entity_id from facility_exposure_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Read legal_entity_id from facility_exposure_snapshot for each facility.
 </v>
       </c>
       <c r="E83" t="str">
@@ -8155,7 +8337,7 @@
         <v>Raw</v>
       </c>
       <c r="J83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_entity_id from facility_exposure_snapshot for each facility as-of reporting date.
+        <v xml:space="preserve">Read legal_entity_id from facility_exposure_snapshot for each facility.
 </v>
       </c>
       <c r="K83" t="str">
@@ -8165,10 +8347,10 @@
         <v>Y</v>
       </c>
       <c r="M83" t="str">
-        <v>Raw</v>
+        <v>Calc</v>
       </c>
       <c r="N83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read legal_entity_id per counterparty.
+        <v xml:space="preserve">Count of distinct booking legal entities per counterparty.
 </v>
       </c>
       <c r="O83" t="str">
@@ -8178,10 +8360,10 @@
         <v>Y</v>
       </c>
       <c r="Q83" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="R83" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_entity_id per L3 desk segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L3 desk segment.
 </v>
       </c>
       <c r="S83" t="str">
@@ -8191,10 +8373,10 @@
         <v>Y</v>
       </c>
       <c r="U83" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="V83" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_entity_id per L2 portfolio segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L2 portfolio segment.
 </v>
       </c>
       <c r="W83" t="str">
@@ -8204,10 +8386,10 @@
         <v>Y</v>
       </c>
       <c r="Y83" t="str">
-        <v>Agg</v>
+        <v>Calc</v>
       </c>
       <c r="Z83" t="str" xml:space="preserve">
-        <v xml:space="preserve">SUM of facility-level legal_entity_id per L1 business segment segment.
+        <v xml:space="preserve">Count of distinct booking legal entities per L1 business segment.
 </v>
       </c>
       <c r="AA83" t="str">
@@ -9803,14 +9985,23 @@
         <v>RSK-002</v>
       </c>
       <c r="B101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Current external credit agency rating assigned to the obligor. Used for benchmarking, regulatory reporting, and external credit risk validation. Sourced based on external Rating provider (S&amp;P, Moodys, Fitch) - populated based on firm's preferred recognized rating provider.
+        <v xml:space="preserve">External credit agency rating expressed as a numeric notch value from the rating_scale_dim. At facility/counterparty levels, returns the raw notch of the external rating. At aggregate levels (desk, portfolio, segment), computes the exposure-weighted average notch across all positions, rounded to the nearest whole notch. Lower notch = better rating (e.g., 1=AAA, 21=D). Sourced from position.external_risk_rating, mapped to rating_scale_dim.rating_value.
 </v>
       </c>
       <c r="C101" t="str">
         <v>Risk Rating - External Rating</v>
       </c>
       <c r="D101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating from position for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+   AND   rs.is_current_flag = 'Y'
+4. COMPUTE
+   metric_value = rs.rating_value
 </v>
       </c>
       <c r="E101" t="str">
@@ -9829,7 +10020,16 @@
         <v>Raw</v>
       </c>
       <c r="J101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating from position for each facility as-of reporting date.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+   WHERE fm.is_active_flag = 'Y'
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+   AND   rs.is_current_flag = 'Y'
+4. COMPUTE
+   metric_value = rs.rating_value
 </v>
       </c>
       <c r="K101" t="str">
@@ -9842,7 +10042,15 @@
         <v>Raw</v>
       </c>
       <c r="N101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Read external_risk_rating per counterparty.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. GROUP BY fm.counterparty_id
+5. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="O101" t="str">
@@ -9852,10 +10060,20 @@
         <v>Y</v>
       </c>
       <c r="Q101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="R101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L3 desk segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+   ON    fm.facility_id = pos.facility_id
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt)
+   ON    ebt.managed_segment_id = fm.lob_segment_id
+5. GROUP BY ebt.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="S101" t="str">
@@ -9865,10 +10083,19 @@
         <v>Y</v>
       </c>
       <c r="U101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="V101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L2 portfolio segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2)
+   Traverse L3 -&gt; L2 via parent_segment_id
+5. GROUP BY ebt_l2.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="W101" t="str">
@@ -9878,10 +10105,19 @@
         <v>Y</v>
       </c>
       <c r="Y101" t="str">
-        <v>Avg</v>
+        <v>Calc</v>
       </c>
       <c r="Z101" t="str" xml:space="preserve">
-        <v xml:space="preserve">AVG of facility-level external_risk_rating per L1 business segment segment.
+        <v xml:space="preserve">1. LOAD  l2.position  (pos)
+   WHERE pos.as_of_date = :as_of_date
+2. JOIN  l2.facility_master  (fm)
+3. LEFT JOIN  l1.rating_scale_dim  (rs)
+   ON    rs.rating_notch = pos.external_risk_rating
+4. LEFT JOIN  l1.enterprise_business_taxonomy  (ebt_l3, ebt_l2, ebt_l1)
+   Traverse L3 -&gt; L2 -&gt; L1 via parent_segment_id chain
+5. GROUP BY ebt_l1.managed_segment_id
+6. COMPUTE
+   metric_value = ROUND(AVG(rating_value))
 </v>
       </c>
       <c r="AA101" t="str">

</xml_diff>